<commit_message>
docs(research): ingest and codify Yin TP Trade b-shape sideway accumulation vs pause video
</commit_message>
<xml_diff>
--- a/docs/research/MASTER_VIDEO_DATABASE.xlsx
+++ b/docs/research/MASTER_VIDEO_DATABASE.xlsx
@@ -479,7 +479,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J45"/>
+  <dimension ref="A1:J46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -562,20 +562,70 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Yin tập trade</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Cách nhận biết giá sideway đang tạo đáy hay phân phối. #trading #trad...</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Cách nhận biết giá sideway đang tạo đáy hay phân phối. #trading #trader #kienthuckinhte #smc</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Nhiều đại vợ Cảm ơn các bạn đã đón xem video này, hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Cảm ơn các bạn đã đón xem video này, hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Cảm ơn các bạn đã đón xem video này, hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Cảm ơn các bạn đã đón xem video này, hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Cảm ơn các bạn đã đón xem video này, hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>1:15</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@yin.tp.trade/video/7694660547685551380</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E3" t="inlineStr">
         <is>
           <t>TradingLab</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>How to Avoid False Breakouts (Avoid The Trap)</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>Quy tắc Phân biệt Fakeout vs Breakout &amp; Bộ lọc Fibonacci Golden Zone:
 1. Fakeout (Phá vỡ giả): Nến chỉ quét râu (wick) qua đỉnh/đáy rồi đóng nến ngược lại bên trong -&gt; Tín hiệu từ chối giá và gom thanh khoản.
@@ -588,7 +638,7 @@
    - Bước 4: Chờ giá hồi về Golden Zone (0.618 - 0.79) mới kích hoạt Buy. SL đặt dưới đáy Fakeout, TP tại đỉnh Breakout. R:R cực cao.</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="H3" t="inlineStr">
         <is>
           <t>What if I told you false breakouts are
 one of the most common ways traders lose
@@ -805,47 +855,47 @@
 inside my Telegram. See you in there.</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>8:00</t>
         </is>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=2yePksvT64I</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" t="n">
-        <v>2</v>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>TradingLab</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>You're Using Liquidity Wrong</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>Quy tắc phân biệt Vùng Cản Thật (Real Zone) và Vùng Mồi Nhử (Inducement Zone):
 1. Vùng B (Inducement): Là đỉnh hồi đầu tiên (minor high/low) sau cú phá vỡ. Nếu phía trên Vùng B còn khoảng trống Imbalance (FVG) chưa lấp, Vùng B 100% là bẫy mồi nhử thanh khoản -&gt; CẤM vào lệnh tại B.
@@ -855,7 +905,7 @@
 5. SL: Đặt trên đỉnh Vùng A. TP: Vùng Demand/Supply đối diện. Tỷ lệ R:R tối ưu đạt 1:5+.</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="H4" t="inlineStr">
         <is>
           <t>[00:00:00] Is this liquidity? Is this liquidity? Is
 [00:00:02] this liquidity? Or is this liquidity? If
@@ -1063,52 +1113,52 @@
 [00:07:45] works for you. See you next time.</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>7:50</t>
         </is>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=RKU7D9PxLgY</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Wysetrade</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="F5" t="inlineStr">
         <is>
           <t>ULTIMATE Supertrend Indicator Trading Strategy (FREE FULL COURSE)</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G5" t="inlineStr">
         <is>
           <t>Khóa học chiến lược Supertrend toàn diện: 1. Tham số chuẩn Factor 2.5 - 3.0 (ATR 10). 2. Không trade tín hiệu đảo chiều độc lập (tránh whipsaw). 3. Quy tắc hợp lưu: Supertrend định hướng Bias + Price Action/Key Levels kích hoạt Entry. 4. Chiến lược Dynamic Trailing Stoploss theo dải Supertrend bắt trọn sóng dài. 5. Bộ lọc đa khung thời gian (HTF Trend Filter).</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="H5" t="inlineStr">
         <is>
           <t>[00:00:00] One of the most effective trading tools
 [00:00:02] is the super trend indicator, but you'd
@@ -1426,52 +1476,52 @@
 [00:12:08] change. Two, you had this key sup</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>17:02</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=As6Sr3OzhzE</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr">
+      <c r="D6" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr">
+      <c r="E6" t="inlineStr">
         <is>
           <t>TRADING RUSH</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr">
+      <c r="F6" t="inlineStr">
         <is>
           <t>How I Increased Win Rate In Trading (WITH PROOF)</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G6" t="inlineStr">
         <is>
           <t>5 Quy tắc tăng Win Rate dựa trên dữ liệu thực nghiệm: 1. Tỷ lệ R:R tối ưu 1.5:1 (Sweet Spot). 2. Đặt TP dưới Swing High khi pullback sâu. 3. Mua sát đáy Support và chốt sớm khi vừa thoát vùng cản. 4. Hạ R:R khi thị trường xấu để bảo vệ vốn. 5. Kiên nhẫn đứng ngoài khi không có setup.</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="H6" t="inlineStr">
         <is>
           <t>[00:00:01] when I started trading around 8 years
 [00:00:03] ago I saw many people giving advice on
@@ -1681,52 +1731,52 @@
 [00:07:42] [Music]</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>7:44</t>
         </is>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=IpSlHWMGgY4</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="2" t="inlineStr">
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr">
+      <c r="D7" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr">
+      <c r="E7" t="inlineStr">
         <is>
           <t>The Trading Channel</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr">
+      <c r="F7" t="inlineStr">
         <is>
           <t>The Only Price Action Trading Video You Will Ever Need (Full Course)</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G7" t="inlineStr">
         <is>
           <t>Khóa học Price Action toàn diện: Xác định cấu trúc thị trường (Market Structure), các vùng Hỗ trợ/Kháng cự chính (Major Support &amp; Resistance), đường Xu hướng (Trendlines), các mô hình nến kích hoạt lệnh (Engulfing, Pin bar) và cách đo lường tỷ lệ R:R tối thiểu 1:2.</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="H7" t="inlineStr">
         <is>
           <t>**`[00:00:00]`** this video currently has over 21 million this video currently has over 21 million views on YouTube and the reason so many views on YouTube and the reason so many views on YouTube and the reason so many Traders found that video valuable is Traders found that video valuable is Traders found that video valuable is because I poured a ton of time and because I poured a ton of time and because I poured a ton of time and effort to ensure that by the end of that.
 **`[00:00:12]`** effort to ensure that by the end of that effort to ensure that by the end of that video Traders knew everything they video Traders knew everything they video Traders knew everything they needed to know about technical analysis needed to know about technical analysis needed to know about technical analysis in this video I'm doing the same exact in this video I'm doing the same exact in this video I'm doing the same exact thing for Price action so throughout the.
@@ -1762,52 +1812,52 @@
 **`[00:04:47]`** this Market to be in an uptrend and this this Market to be in an uptrend and this process just continues as we go higher process just continues as we go higher process just continues as we go higher this move here we go from the low of our this move here we go from the low of our this move here we go from the low of our pullback we break and close above that pullback we break and close a</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>47:16</t>
         </is>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=td5TjsqDCKw</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="2" t="inlineStr">
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 2 (Mới thêm - Khóa học 2.5h)</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
+      <c r="D8" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E7" t="inlineStr">
+      <c r="E8" t="inlineStr">
         <is>
           <t>Jason Graystone</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr">
+      <c r="F8" t="inlineStr">
         <is>
           <t>Trading for Beginners Part 1 - FULL TRADING COURSE TUTORIAL</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G8" t="inlineStr">
         <is>
           <t>Khóa học Trading cơ bản đến nâng cao 2.5 giờ: Bản chất thị trường tài chính, quản lý rủi ro và vốn (Risk Management 1%), toán học xác suất trong trading, xây dựng kế hoạch giao dịch (Trading Plan), tâm lý kỷ luật và nhật ký giao dịch.</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="H8" t="inlineStr">
         <is>
           <t>**`[00:00:00]`** all right welcome to the video this is all right welcome to the video this is trading for beginners or trading for trading for beginners or trading for trading for beginners or trading for dummies as the thumbnail says and the dummies as the thumbnail says and the dummies as the thumbnail says and the goal of this video is to get you from goal of this video is to get you from goal of this video is to get you from struggling or zero profits or complete.
 **`[00:00:10]`** struggling or zero profits or complete struggling or zero profits or complete beginner right through to consistently beginner right through to consistently beginner right through to consistently profitable Trader which means it's a profitable Trader which means it's a profitable Trader which means it's a comp like complete and comprehensive comp like complete and comprehensive comp like complete and comprehensive program all in itself which means it's.
@@ -1843,52 +1893,52 @@
 **`[00:04:16]`** question of what's the real deal and not question of what's the real deal and not only that you'll learn so much in this only that you'll learn so much in this only that you'll learn so much in this lesson that you won't need to go and lesson that yo</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>2:26:39</t>
         </is>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=_YVQN6_nkfs</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" t="inlineStr">
+    <row r="9">
+      <c r="A9" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>🔴 ƯU TIÊN 1 (Mới thêm - Xem ngay)</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>2026-10-15</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr">
+      <c r="D9" t="inlineStr">
         <is>
           <t>YouTube</t>
         </is>
       </c>
-      <c r="E8" t="inlineStr">
+      <c r="E9" t="inlineStr">
         <is>
           <t>Rayner Teo</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr">
+      <c r="F9" t="inlineStr">
         <is>
           <t>The Ultimate Candlestick Patterns Trading Course (Khóa Học Nến Toàn Diện)</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G9" t="inlineStr">
         <is>
           <t>Hệ thống T.A.E Framework (Trend - Area of Value - Entry Trigger), kỹ thuật gộp nến đa khung (2 nến 1h = 1 nến Pin bar 2h), mô hình nến Engulfing, Hammer, Shooting Star, Morning/Evening Star, Tweezer. Quy tắc không trade nến độc lập mà phải tại cản/MA động.</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="H9" t="inlineStr">
         <is>
           <t># TOÀN BỘ SCRIPT (LỜI THOẠI) KHÓA HỌC: THE ULTIMATE CANDLESTICK PATTERNS TRADING COURSE
 - **Kênh YouTube:** [Rayner Teo (@tradingwithrayner)](https://www.youtube.com/@tradingwithrayner)
@@ -1953,64 +2003,14 @@
 **`[00:11:47]`** did close higher above the first so if you look at it this second candle over here it it closed higher above this one over here so that's why you got a bullish bullish close okay and similar for this right this candle it closed right but it didn't exceed the open of this candle so that's why it's still red on the two hour ti</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>38:10</t>
         </is>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>https://www.youtube.com/watch?v=C3KRwfj9F8Q</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>🟡 Ưu tiên 2 (Cốt lõi SMC/ICT)</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>Vnrebates</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>Khám Phá Setup Giao Dịch Của Trader Nhận Payout 2 Triệu USD</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>SMC &amp; ICT: Setup phiên Á - Âu quét thanh khoản, 4 tiêu chí khối Order Block chuẩn (BOS, FVG, Premium/Discount, Sweep), Fibonacci OTE 0.618 - 0.786 lồng ghép FVG, giáo trình FVG 11 phút.</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>Đây là xét óp giúp Trader Can Pay Out gần 2 triệu đô từ ProfFirm. Chị tôi vai! Lấy giây bút ra ghi nè. Đầu tiên, chờ phiền Á kết thúc, đánh giấu đỉnh và đáy phiền Á. Kích theo, chờ 1 trong 2 vị trí này bị quét. Ở đây, đáy phiền Á đã bị quét. Vào khung M1, chờ phiền Âu mở cửa. Sau khi phiền Âu bắt đầu, giá đóng cửa tạo CISD. Vào lạnh mùa, Stop Loss dứa đáy vừa quét, thê pe ở đỉnh phiền Á. Nhưng nhớ quản lý lạnh, chốt 1 nữa ở đỉnh củ. Ông đã thử xét óp phiền Á này chưa? Comment cho tôi biết nhé!</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>1m - 11m</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>https://www.tiktok.com/@vn_rebates/video/7696474697961196808</t>
         </is>
       </c>
     </row>
@@ -2040,7 +2040,7 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>Thế Nào Là Một Khối Order Block (OB) Chất Lượng</t>
+          <t>Khám Phá Setup Giao Dịch Của Trader Nhận Payout 2 Triệu USD</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Giả chạp OrderBlock rồi, mua được chưa ông? Thử đi! Sao kỳ với ta? Để tôi chỉ ông cách chọn ra OrderBlock chất lượng, sẽ cần những yếu tố gì. 1. OrderBlock đó phải tạo ra phá vỡ câu trúc BRS. 2. Theo sau OrderBlock, phải có 1 app Vega. 3. OrderBlock nằm ở vùng premium cho lệnh bán hoặc discount cho lệnh mua. Ở đây, OrderBlock giảm nằm ở premium. 4. Có quét thanh khoảng trước khi giá hồi về OrderBlock. Chỉ vào lệnh khi OrderBlock có ít nhất 3 trên 4 yếu tố. Vào lệnh bán tại OrderBlock, stoplock trên đỉnh OrderBlock RR12. Anh chọp TP luôn! Ông có chọn OrderBlock theo 4 yếu tố này chưa? Comment cho tôi biết nhé!</t>
+          <t>Đây là xét óp giúp Trader Can Pay Out gần 2 triệu đô từ ProfFirm. Chị tôi vai! Lấy giây bút ra ghi nè. Đầu tiên, chờ phiền Á kết thúc, đánh giấu đỉnh và đáy phiền Á. Kích theo, chờ 1 trong 2 vị trí này bị quét. Ở đây, đáy phiền Á đã bị quét. Vào khung M1, chờ phiền Âu mở cửa. Sau khi phiền Âu bắt đầu, giá đóng cửa tạo CISD. Vào lạnh mùa, Stop Loss dứa đáy vừa quét, thê pe ở đỉnh phiền Á. Nhưng nhớ quản lý lạnh, chốt 1 nữa ở đỉnh củ. Ông đã thử xét óp phiền Á này chưa? Comment cho tôi biết nhé!</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -2060,7 +2060,7 @@
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vn_rebates/video/7696091260565769490</t>
+          <t>https://www.tiktok.com/@vn_rebates/video/7696474697961196808</t>
         </is>
       </c>
     </row>
@@ -2090,7 +2090,7 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Fibonacci OTE Trong Forex: Cách Chọn Điểm Vào Lệnh An Toàn</t>
+          <t>Thế Nào Là Một Khối Order Block (OB) Chất Lượng</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Gia phá đỉnh rồi quay về tét đỉnh con nén en-gu-fing mua thôi! Quang, nếu mua ở đây mà đặt stop-loss ngay dưới vùng đỉnh cũ thì rất không an toàn. Còn nếu đặt stop-loss dưới đấy thì rơ rơ lại rất thấp. Xem nè! Trời ơi, dính stop-loss rồi! Vậy phải làm sao hả ông? Bấu chốt là chúng ta phải tìm được điểm entry có stop-loss an toàn và rơ rơ tốt. Dùng Fibo OTE, kéo từ đáy lên đỉnh theo sưu hướng tăng. Lúc này, ông thấy vùng OTE từ 0.705 đến 0.79 trùng với FVG. Entry ở đây, stop-loss dưới đấy vẫn an toàn mà rơ rơ tốt hơn nhiều. Ông đã biết dùng OTE kết hợp FVG chưa? Comment cho tôi biết nhé!</t>
+          <t>Giả chạp OrderBlock rồi, mua được chưa ông? Thử đi! Sao kỳ với ta? Để tôi chỉ ông cách chọn ra OrderBlock chất lượng, sẽ cần những yếu tố gì. 1. OrderBlock đó phải tạo ra phá vỡ câu trúc BRS. 2. Theo sau OrderBlock, phải có 1 app Vega. 3. OrderBlock nằm ở vùng premium cho lệnh bán hoặc discount cho lệnh mua. Ở đây, OrderBlock giảm nằm ở premium. 4. Có quét thanh khoảng trước khi giá hồi về OrderBlock. Chỉ vào lệnh khi OrderBlock có ít nhất 3 trên 4 yếu tố. Vào lệnh bán tại OrderBlock, stoplock trên đỉnh OrderBlock RR12. Anh chọp TP luôn! Ông có chọn OrderBlock theo 4 yếu tố này chưa? Comment cho tôi biết nhé!</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
@@ -2110,7 +2110,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vn_rebates/video/7695729577947155720</t>
+          <t>https://www.tiktok.com/@vn_rebates/video/7696091260565769490</t>
         </is>
       </c>
     </row>
@@ -2140,7 +2140,7 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Hướng Dẫn Toàn Diện Về Fair Value Gap (FVG)</t>
+          <t>Fibonacci OTE Trong Forex: Cách Chọn Điểm Vào Lệnh An Toàn</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2150,7 +2150,7 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Hôm nay sẽ là 1 video khá là dài Mình sẽ hướng dẫn cho anh em những cái thứ chi tiết và thật chiến nhất về FVG, 1 công cụ cực kìa bánh mẽ trong phương pháp ICT Đầu tiên FVG sẽ được chia hình 4 loại hả? Dạy đầu tiên mà chúng ta sẽ học, đó chính là FVG Breakaway Nó sẽ được hình thành từ 3 cái nến tăng liên tiếp với anh em Và nó sẽ là dạy mở rộng Thì khi anh em thấy xuất hiện 3 cái nến tăng liên tiếp Hình thành 1 cái FVG Nó báo hiệu 1 cái động lực tăng mạnh của thị trường Và khả năng cái nha, khả năng cao Những cái FVG Breakaway này á Đến 80% giá nó sẽ tăng tiếp tục Và nó không quay về test cái FVG Thói chúng ta sẽ xem bí dụ mà Ở đây chúng ta có Cây nến khung H1 Anh em thấy không? Đây là 3 cây nến tăng liên tiếp Và nó tạo ra 1 cái buồn FVG ở đây Đúng không? Thì anh em quay xác anh em thấy được đỏ ràng là Giá đó không có test về cái FVG này Ở đây cũng có rất nhiều trường hợp như vậy hả? Này nè mình Khi nó tạo ra 1 cái FVG Breakaway á Ở đây nè Anh em thấy không? Thì giá nó liên tiếp tục tăng lên, tăng lên, tăng lên Cho đến ngày hôm sau nó mới quay về test Mà khi mà nó đi xa như vậy nó quay về test Thì nó không còn mạnh nữa Những FVG được tạo ra thì chúng ta sẽ muốn nó phải test liền Thì khi anh em thấy FVG Breakaway như thế này nè Thì anh em sẽ phải vào trong khung M5 Để anh em tìm kiếm những lệnh tiếp diễn Ok, mình sẽ vào trong khung M5 Mình vào trong khung M5 nè Rồi, mình sẽ tui vào chỗ này Thì trong khung M5 nó lại tiếp tục tạo ra 1 cái FVG Đúng không? Ở đây Thì bây giờ anh em có thể follow hell cái FVG mở năm này rồi Tại vì khi mà nó tạo ra FVG Breakaway ở khung H1 Thì trong khung M5 nó cũng sẽ tạo 1 cái động lực tăng Và lúc này anh em chỉ cần mua ở cái FVG trong khung M5 là được Rồi chúng ta cùng xem giá chạy ha Giá quay về test cái FVG trong khung M5 nè Mà tăng lên Đó chính là cách mà chúng ta sẽ giao dịch với FVG Breakaway Tiếp tục mình sẽ đến với 1 cái FVG bình thường Đó là 1 cái FVG có 2 cái nến tăng và 1 cái nến giảm như thế này Nó không phải là dẹn mở rộng anh em ha Thì với cái FVG dẹn này Giá nó có khả năng test lại cái FVG Sau đó mới tăng ha Thì chúng ta sẽ cùng vào trong cái bí dụ của EU dưới đây Thì bí bí EU này sẽ khá ngược lại là sẽ gồm là 2 cái nến giảm và 1 cái nến tăng Thì nó là FVG dẹn thường nhưng mà nằm trong xuống giảm anh em ha Thì chúng ta cũng có 1 cái FVG chỗ này Mình sẽ đặt lên nó là FVG H1 đi Cho anh em dễ quay xác rồi Rồi bây giờ mình sẽ vào trong khung M5 Tại vì đây là FVG dẹn thường, không phải là dẹn Breakaway Thì giá có khả năng sẽ test lại ha Vào trong khung M5 Rồi mình chờ test lại cái FVG này Rồi thì khi nó test lại cái FVG này rồi Nhưng mà M5 vẫn đang là 1 cái xuống dẹn này, 1 xuống tăng ha Thì mình sẽ chờ nó phá vào cái đáy này Rồi thì khi nó phá vào cái đáy này Nó hình thành cho mình 1 cái FVG Mở 5 ở đây, đúng chưa? Mình sẽ NG ở cái FVG mở 5 này Đặt stop-lock ở trên đây Và đặt cái mức tê bê là 2R 2R này mà Cùng sẽ nhá nó chạy ha Giá test lại cái FVG này Và sạch xuống, đó chính là cách chúng ta ứng dụng FVG bình thường ha Rồi tiếp tục 1 vàng FVG nữa Đó là EFVG Cũng tương tự như thế này, chúng ta có 1 cái FVG tăng đúng không? Đây Và nếu như cái FVG tăng này Nó bị phá bởi 1 cái nến Thay là nhiều cái nến nhứng chìm ha Nó chung là nhứng chìm cái FVG Như thế này Đó Nhứng chìm ha Thì cái FVG này Nó sẽ không còn là FVG nữa Nhưng mà nó sẽ là EFVG Nó sẽ trành EFVG Thì với EFVG, nghĩa là 1 cái FVG bị nhứng chìm Chúng ta sẽ chờ nó test lại và xeo xuống Hoặc là nếu như nó tạo 3 cái nến giảm Mà 1 cái nến tăng nhứng chìm thì chúng ta sẽ bài lên ha Tương tự chúng ta có 1 cái bí vụ ở đây Thử này ha Đây là 3 cái nến giảm đúng chưa? 3 cái nến giảm 1, 2, 3 Nó tạo chúng ta 1 cái FVG Đúng không? Và cái FVG này đã bị nhứng chìm Bởi cái nến tăng này Thì chỗ này nó sẽ trở thành EFVG Rồi cái nhiệm vụ chúng ta chỉ là vì 3 lại khi giá test cái EFVG Đã X lời dưới đây và tề bên trên Rồi cùng xem giá chạy đẹp Giá test lại cái EFVG và Tiếp tục tăng lên Đó là cách xài EFVG ha Rồi 1 dạng FVG nữa Đó là B rồi B B được đựng dễ như thế nào Nếu dư Mình sẽ kéo 3 cái nến giảm Chưa có 3 cái nữa này đi Thì chúng ta sẽ có 1 cái FVG tăng đúng không? Nhưng nếu như cái FVG tăng này Bị nhứng chìm bởi 1 cái FVG giảm đối diện Đây, trái hẹn như thế này là 1 cái 3 cái nến giảm đúng không? 3 cái nến giảm này tạo 1 cái FVG đối diện ở đây Đúng chưa? Đó Thì đây gọi là B rồi B Hay gọi là Subton ha Đây là cái dạng mạnh nha ném Dạng mạnh của FVG đảo chiều Tại vì khi mà Nên nó biết là khi mà giá tạo 1 FVG Chứng đó động lực tăng nó rất là mạnh đúng không? Nhưng mà nó lại bị nhứng chìm Bởi 1 cái động lực giảm Chứng tạo là tại cái vị trí này nha Là cái bên bán nó nhảy vào rất mạnh Thì anh em sẽ canh nó test lại cái FVG này Để anh em bán xuống ha Đó chính là Subton Thì gọi là B rồi B Rồi chúng ta sẽ cùng nhau Nhìn vào cái ví dụ con HU với đây Đây Sau khi giá nó sang ra hành khoảng cái đỉnh bên đây Nè em thấy không? Này nó sang hành khoảng cái đỉnh nè Mình sẽ tua lại ha Nó sang hành khoảng cái đỉnh xong Nó tạo chúng ta 1 cái FVG Đúng chưa? FVG Rồi Và FVG này bị diễn em Bị nhứng chìm bởi cái FVG đối diện Chính là cái FVG này Đúng không? Này FVG tăng bị nhứng chìm bởi FVG giảm Sau đó nó test lại bằng cái nánh này Đây cái nánh này Khi nó tạo được cái FVG giảm nhứng chìm rồi Thì chúng ta tham cú Subton rồi Thì anh em sẽ đặt 1 cái lệnh cell Ngay tại cái FVG giảm được tạo ra X lời đặt trên đây Và TB TB về đáy gần nhất Chính là vị trí này Rồi cùng xem giá chạy ha Giá test lại Và sắp mạnh xuống ha Đó chính là Subton Bây giờ mình nói là khi sẽ là Subton Giá đi rất là mạnh đúng không? Nó sắp rất là mạnh ha Rồi tiếp tục Chúng ta đến với cái FVG Cuối cùng Cái FVG này không dùng để vào lệnh Mà FVG này dùng để làm gì anh em? Dùng để làm đến TB Làm đến TB ha Hay còn gọi là ReFVG ReFVG Nghĩa là sao? Nghĩa là Đây là cái điểm mà anh em sẽ chốt lời Cái điểm này sẽ chốt lời Nếu như anh em có lệnh mua Thì nếu như anh em có 1 cái lệnh mua ở đây Mình giả sử ở đây là 1 case FVG Đúng không? Anh em mua ở đây Anh em phải tới bệp đầu Tên bệp đầu thì đương nhiên là chúng ta sẽ Nhìn những cái cản rồi Thì ở đây có 1 cái FVG đói diện nữa nào Đúng không? Một cái FVG nó diễn nữa Thì nếu như anh em mua ở đây Anh em có thể TB ở đây Và nếu như nó lụng ở đây Thì nó sẽ lên đầu Nó sẽ tìm kiếm ở đâu tiếp Nó sẽ tìm kiếm cái FVG trên đây Thì cái FVG này cũng gọi là ReFVG luôn Và cái FVG này cũng gọi là ReFVG Cả hai cái này đều là ReFVG ha Tao cùng xem giá nó chạy tiếp Nó thì khi giá nó Nó lại tiếp tục Test về cái FVG này Đúng không? Đó tiện em có thể mua ha Có thể mua lên từ đây Rồi giá nó tiếp tục tăng lên thôi Rồi thì TB của này sẽ lâu TB này sẽ là cái ReFVG này Ở chỗ này nó cũng sẽ có 1 cái FVG nào Anh em cũng có thể mua ở cái FVG này Hét lờ dưới đây Và TB cũng về cái ReFVG luôn Hai lần chúng ta được TB về cái ReFVG này Và nếu em kia giá nó chạm đến cái ReFVG này ha Nó sẽ có phản ứng mạnh Mình không biết là nó có xuyên được cái FVG này không Hay là từ cái ReFVG này nó sẽ đảo chiều Nhưng đây là cái điểm TB đẹp nhất Đó thì đây là cái ứng dụng của ReFVG ha Rồi thì trong video hôm nay mình đã chia sẻ cho anh em Hết tất cả những các loại ReFVG có trên thị trường Hầu tiên là ReqAway ReFVG ReFVG bình thường ReFVG BW Và ReFVG Đó là những loại ReFVG mà anh em cần biết Để có thể áp dụng nó vào trong cái quá trình trái đình của mình ha Ok cám ơn em đã theo dõi video này Và nếu anh em thấy hay Các bạn có thể lưu video và bấm vào cái link bio Để tiếp cận những phương pháp trái đình hiệu quả nhất ha Ok cám ơn em đã theo dõi video</t>
+          <t>Gia phá đỉnh rồi quay về tét đỉnh con nén en-gu-fing mua thôi! Quang, nếu mua ở đây mà đặt stop-loss ngay dưới vùng đỉnh cũ thì rất không an toàn. Còn nếu đặt stop-loss dưới đấy thì rơ rơ lại rất thấp. Xem nè! Trời ơi, dính stop-loss rồi! Vậy phải làm sao hả ông? Bấu chốt là chúng ta phải tìm được điểm entry có stop-loss an toàn và rơ rơ tốt. Dùng Fibo OTE, kéo từ đáy lên đỉnh theo sưu hướng tăng. Lúc này, ông thấy vùng OTE từ 0.705 đến 0.79 trùng với FVG. Entry ở đây, stop-loss dưới đấy vẫn an toàn mà rơ rơ tốt hơn nhiều. Ông đã biết dùng OTE kết hợp FVG chưa? Comment cho tôi biết nhé!</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -2160,7 +2160,7 @@
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vn_rebates/video/7474060511584324885</t>
+          <t>https://www.tiktok.com/@vn_rebates/video/7695729577947155720</t>
         </is>
       </c>
     </row>
@@ -2190,7 +2190,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Xác Định Thanh Khoản Thị Trường (Liquidity ICT)</t>
+          <t>Hướng Dẫn Toàn Diện Về Fair Value Gap (FVG)</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2200,7 +2200,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>ICT đã từng nói, tị trường chỉ làm có 2 việc thôi Thứ nhất là quay thanh khỏe và thứ 2 là lắp này các FVG Điều này có nghĩa là nếu như anh em vào một cái lệnh nào đó mà anh em chưa tìm nấy thanh khỏe thì rất có thể anh em sẽ trở thành thanh khỏe ICT là một trader với quan điểm dâu dịch là tị trường luôn luôn tìm thanh khỏe trước khi có những bước đi tiếp theo Thì sau khi tham khảo vào cái tư duy của ICT thì mình đã rút ra được một số các bài học và hôm nay mình sẽ chia sẻ anh em để có thể tăng thêm một cái tự lời hắn của mình Ok, nè Ma, thì anh em nhìn 2 cái bí vụ với đây thì anh em thấy khi giá nó phải hướng tới một cái buồn giá nào đó thì sẽ có 2 trường hợp xảy ra đúng không? Một là giá chạm đứng cái buồn này và tăng lên Nếu anh em ba này sẽ thắng Còn hai, nó chạm buồn này nhưng mà nó không tăng mà nó xuyên luôn thì anh em sẽ thua Anh em nghĩ là chỉ có 2 trường hợp thôi hả? Còn 1 trường hợp nữa đó là giá nó vét đáy xong nó mới thanh Đó Vậy thì nếu như anh em chọn 1 cái chờ về đây anh em ba lên thì anh em có tới 2 trường hợp mà anh em có thể thua được và là cái này và cái này Vậy thì thông bình hơn nó sẽ chờ cái gì? Ta sẽ chờ giá nó vét xong rồi chúng ta mới bầu lệnh thì lúc đó anh em có thể loại được bớt thêm 1 trường hợp thua nữa thì cái thể thắng nó sẽ tăng lên đúng không? Rồi bây giờ nó sẽ cùng nhau nhìn vào cái trạng này Đây là 1 cái cấu chút tăng đúng rồi anh em, chút tăng này thì có nhiều nên sẽ canh 3 cái giá qua bên bùn đáy này Thì khi giá trạm bùn đáy này nó sức hiểm cơ nến bin ba đứt rau thì là phần anh em sẽ vào buồn ở đây x lờ dưới cái đáy này và bề bề thì chúng ta cùng xem giá nó đi như thế nào hả? Mới vụng ta 1 vài trành bị x lờ sau đó nó mới tăng lên thì mình sẽ vào lệnh khi này bị béc rồi và tiếp tục tăng lên nè sau khi béc xong anh em phải tăng lên nó đóng đến qua cái nến này thì lúc này đây chỉ là 1 cái phá bởi giả thôi nè thì chúng ta mới bắt đầu vào lệnh mua vị trí này đạt sublots như đây và tb lên trần cùng xem giá nó chạy hả? Sau khi được bấy đựng sublots rồi thì giá nó đi rất là nhanh và đạt được tb đó là cách để thông minh nhớ nè chờ giá quá thân ngoại thông chúng ta mới vào chúng ta sẽ có tự lệnh hắn cao hơn ok nè mà lô video lại để xem kì cứng thiết</t>
+          <t>Hôm nay sẽ là 1 video khá là dài Mình sẽ hướng dẫn cho anh em những cái thứ chi tiết và thật chiến nhất về FVG, 1 công cụ cực kìa bánh mẽ trong phương pháp ICT Đầu tiên FVG sẽ được chia hình 4 loại hả? Dạy đầu tiên mà chúng ta sẽ học, đó chính là FVG Breakaway Nó sẽ được hình thành từ 3 cái nến tăng liên tiếp với anh em Và nó sẽ là dạy mở rộng Thì khi anh em thấy xuất hiện 3 cái nến tăng liên tiếp Hình thành 1 cái FVG Nó báo hiệu 1 cái động lực tăng mạnh của thị trường Và khả năng cái nha, khả năng cao Những cái FVG Breakaway này á Đến 80% giá nó sẽ tăng tiếp tục Và nó không quay về test cái FVG Thói chúng ta sẽ xem bí dụ mà Ở đây chúng ta có Cây nến khung H1 Anh em thấy không? Đây là 3 cây nến tăng liên tiếp Và nó tạo ra 1 cái buồn FVG ở đây Đúng không? Thì anh em quay xác anh em thấy được đỏ ràng là Giá đó không có test về cái FVG này Ở đây cũng có rất nhiều trường hợp như vậy hả? Này nè mình Khi nó tạo ra 1 cái FVG Breakaway á Ở đây nè Anh em thấy không? Thì giá nó liên tiếp tục tăng lên, tăng lên, tăng lên Cho đến ngày hôm sau nó mới quay về test Mà khi mà nó đi xa như vậy nó quay về test Thì nó không còn mạnh nữa Những FVG được tạo ra thì chúng ta sẽ muốn nó phải test liền Thì khi anh em thấy FVG Breakaway như thế này nè Thì anh em sẽ phải vào trong khung M5 Để anh em tìm kiếm những lệnh tiếp diễn Ok, mình sẽ vào trong khung M5 Mình vào trong khung M5 nè Rồi, mình sẽ tui vào chỗ này Thì trong khung M5 nó lại tiếp tục tạo ra 1 cái FVG Đúng không? Ở đây Thì bây giờ anh em có thể follow hell cái FVG mở năm này rồi Tại vì khi mà nó tạo ra FVG Breakaway ở khung H1 Thì trong khung M5 nó cũng sẽ tạo 1 cái động lực tăng Và lúc này anh em chỉ cần mua ở cái FVG trong khung M5 là được Rồi chúng ta cùng xem giá chạy ha Giá quay về test cái FVG trong khung M5 nè Mà tăng lên Đó chính là cách mà chúng ta sẽ giao dịch với FVG Breakaway Tiếp tục mình sẽ đến với 1 cái FVG bình thường Đó là 1 cái FVG có 2 cái nến tăng và 1 cái nến giảm như thế này Nó không phải là dẹn mở rộng anh em ha Thì với cái FVG dẹn này Giá nó có khả năng test lại cái FVG Sau đó mới tăng ha Thì chúng ta sẽ cùng vào trong cái bí dụ của EU dưới đây Thì bí bí EU này sẽ khá ngược lại là sẽ gồm là 2 cái nến giảm và 1 cái nến tăng Thì nó là FVG dẹn thường nhưng mà nằm trong xuống giảm anh em ha Thì chúng ta cũng có 1 cái FVG chỗ này Mình sẽ đặt lên nó là FVG H1 đi Cho anh em dễ quay xác rồi Rồi bây giờ mình sẽ vào trong khung M5 Tại vì đây là FVG dẹn thường, không phải là dẹn Breakaway Thì giá có khả năng sẽ test lại ha Vào trong khung M5 Rồi mình chờ test lại cái FVG này Rồi thì khi nó test lại cái FVG này rồi Nhưng mà M5 vẫn đang là 1 cái xuống dẹn này, 1 xuống tăng ha Thì mình sẽ chờ nó phá vào cái đáy này Rồi thì khi nó phá vào cái đáy này Nó hình thành cho mình 1 cái FVG Mở 5 ở đây, đúng chưa? Mình sẽ NG ở cái FVG mở 5 này Đặt stop-lock ở trên đây Và đặt cái mức tê bê là 2R 2R này mà Cùng sẽ nhá nó chạy ha Giá test lại cái FVG này Và sạch xuống, đó chính là cách chúng ta ứng dụng FVG bình thường ha Rồi tiếp tục 1 vàng FVG nữa Đó là EFVG Cũng tương tự như thế này, chúng ta có 1 cái FVG tăng đúng không? Đây Và nếu như cái FVG tăng này Nó bị phá bởi 1 cái nến Thay là nhiều cái nến nhứng chìm ha Nó chung là nhứng chìm cái FVG Như thế này Đó Nhứng chìm ha Thì cái FVG này Nó sẽ không còn là FVG nữa Nhưng mà nó sẽ là EFVG Nó sẽ trành EFVG Thì với EFVG, nghĩa là 1 cái FVG bị nhứng chìm Chúng ta sẽ chờ nó test lại và xeo xuống Hoặc là nếu như nó tạo 3 cái nến giảm Mà 1 cái nến tăng nhứng chìm thì chúng ta sẽ bài lên ha Tương tự chúng ta có 1 cái bí vụ ở đây Thử này ha Đây là 3 cái nến giảm đúng chưa? 3 cái nến giảm 1, 2, 3 Nó tạo chúng ta 1 cái FVG Đúng không? Và cái FVG này đã bị nhứng chìm Bởi cái nến tăng này Thì chỗ này nó sẽ trở thành EFVG Rồi cái nhiệm vụ chúng ta chỉ là vì 3 lại khi giá test cái EFVG Đã X lời dưới đây và tề bên trên Rồi cùng xem giá chạy đẹp Giá test lại cái EFVG và Tiếp tục tăng lên Đó là cách xài EFVG ha Rồi 1 dạng FVG nữa Đó là B rồi B B được đựng dễ như thế nào Nếu dư Mình sẽ kéo 3 cái nến giảm Chưa có 3 cái nữa này đi Thì chúng ta sẽ có 1 cái FVG tăng đúng không? Nhưng nếu như cái FVG tăng này Bị nhứng chìm bởi 1 cái FVG giảm đối diện Đây, trái hẹn như thế này là 1 cái 3 cái nến giảm đúng không? 3 cái nến giảm này tạo 1 cái FVG đối diện ở đây Đúng chưa? Đó Thì đây gọi là B rồi B Hay gọi là Subton ha Đây là cái dạng mạnh nha ném Dạng mạnh của FVG đảo chiều Tại vì khi mà Nên nó biết là khi mà giá tạo 1 FVG Chứng đó động lực tăng nó rất là mạnh đúng không? Nhưng mà nó lại bị nhứng chìm Bởi 1 cái động lực giảm Chứng tạo là tại cái vị trí này nha Là cái bên bán nó nhảy vào rất mạnh Thì anh em sẽ canh nó test lại cái FVG này Để anh em bán xuống ha Đó chính là Subton Thì gọi là B rồi B Rồi chúng ta sẽ cùng nhau Nhìn vào cái ví dụ con HU với đây Đây Sau khi giá nó sang ra hành khoảng cái đỉnh bên đây Nè em thấy không? Này nó sang hành khoảng cái đỉnh nè Mình sẽ tua lại ha Nó sang hành khoảng cái đỉnh xong Nó tạo chúng ta 1 cái FVG Đúng chưa? FVG Rồi Và FVG này bị diễn em Bị nhứng chìm bởi cái FVG đối diện Chính là cái FVG này Đúng không? Này FVG tăng bị nhứng chìm bởi FVG giảm Sau đó nó test lại bằng cái nánh này Đây cái nánh này Khi nó tạo được cái FVG giảm nhứng chìm rồi Thì chúng ta tham cú Subton rồi Thì anh em sẽ đặt 1 cái lệnh cell Ngay tại cái FVG giảm được tạo ra X lời đặt trên đây Và TB TB về đáy gần nhất Chính là vị trí này Rồi cùng xem giá chạy ha Giá test lại Và sắp mạnh xuống ha Đó chính là Subton Bây giờ mình nói là khi sẽ là Subton Giá đi rất là mạnh đúng không? Nó sắp rất là mạnh ha Rồi tiếp tục Chúng ta đến với cái FVG Cuối cùng Cái FVG này không dùng để vào lệnh Mà FVG này dùng để làm gì anh em? Dùng để làm đến TB Làm đến TB ha Hay còn gọi là ReFVG ReFVG Nghĩa là sao? Nghĩa là Đây là cái điểm mà anh em sẽ chốt lời Cái điểm này sẽ chốt lời Nếu như anh em có lệnh mua Thì nếu như anh em có 1 cái lệnh mua ở đây Mình giả sử ở đây là 1 case FVG Đúng không? Anh em mua ở đây Anh em phải tới bệp đầu Tên bệp đầu thì đương nhiên là chúng ta sẽ Nhìn những cái cản rồi Thì ở đây có 1 cái FVG đói diện nữa nào Đúng không? Một cái FVG nó diễn nữa Thì nếu như anh em mua ở đây Anh em có thể TB ở đây Và nếu như nó lụng ở đây Thì nó sẽ lên đầu Nó sẽ tìm kiếm ở đâu tiếp Nó sẽ tìm kiếm cái FVG trên đây Thì cái FVG này cũng gọi là ReFVG luôn Và cái FVG này cũng gọi là ReFVG Cả hai cái này đều là ReFVG ha Tao cùng xem giá nó chạy tiếp Nó thì khi giá nó Nó lại tiếp tục Test về cái FVG này Đúng không? Đó tiện em có thể mua ha Có thể mua lên từ đây Rồi giá nó tiếp tục tăng lên thôi Rồi thì TB của này sẽ lâu TB này sẽ là cái ReFVG này Ở chỗ này nó cũng sẽ có 1 cái FVG nào Anh em cũng có thể mua ở cái FVG này Hét lờ dưới đây Và TB cũng về cái ReFVG luôn Hai lần chúng ta được TB về cái ReFVG này Và nếu em kia giá nó chạm đến cái ReFVG này ha Nó sẽ có phản ứng mạnh Mình không biết là nó có xuyên được cái FVG này không Hay là từ cái ReFVG này nó sẽ đảo chiều Nhưng đây là cái điểm TB đẹp nhất Đó thì đây là cái ứng dụng của ReFVG ha Rồi thì trong video hôm nay mình đã chia sẻ cho anh em Hết tất cả những các loại ReFVG có trên thị trường Hầu tiên là ReqAway ReFVG ReFVG bình thường ReFVG BW Và ReFVG Đó là những loại ReFVG mà anh em cần biết Để có thể áp dụng nó vào trong cái quá trình trái đình của mình ha Ok cám ơn em đã theo dõi video này Và nếu anh em thấy hay Các bạn có thể lưu video và bấm vào cái link bio Để tiếp cận những phương pháp trái đình hiệu quả nhất ha Ok cám ơn em đã theo dõi video</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -2210,7 +2210,7 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@vn_rebates/video/7446381153868598534</t>
+          <t>https://www.tiktok.com/@vn_rebates/video/7474060511584324885</t>
         </is>
       </c>
     </row>
@@ -2220,7 +2220,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>🟢 Ưu tiên 3 (Thực chiến Price Action)</t>
+          <t>🟡 Ưu tiên 2 (Cốt lõi SMC/ICT)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2235,32 +2235,32 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>SO Trading</t>
+          <t>Vnrebates</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>3 lỗi vào lệnh khiến bạn bị cắt lỗ oan (và cách sửa) Sửa lỗi quan trọ...</t>
+          <t>Xác Định Thanh Khoản Thị Trường (Liquidity ICT)</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>3 lỗi vào lệnh khiến bạn bị cắt lỗ oan (và cách sửa) Sửa lỗi quan trọng hơn tìm phương pháp mới. 3 lỗi hay gặp: tin tín hiệu khung nhỏ mà quên khung lớn, vào lệnh ngược để gỡ, đóng lệnh vì giá lình xình. Nguồn: nội dung do SO TRADING tự biên soạn. #Shorts #Trading</t>
+          <t>SMC &amp; ICT: Setup phiên Á - Âu quét thanh khoản, 4 tiêu chí khối Order Block chuẩn (BOS, FVG, Premium/Discount, Sweep), Fibonacci OTE 0.618 - 0.786 lồng ghép FVG, giáo trình FVG 11 phút.</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Bị cắt lỗ oan liên tục, có thể lỗi nằm ở chính bạn, không phải phương pháp. Mới giao dịch, ai cũng đi tìm phương pháp tốt nhất. Nhưng sửa từng lỗi sai của mình còn quan trọng hơn nhiều. Lỗi thứ nhất: Thấy tín hiệu đẹp ở khung M5 mà quên nhìn khung lớn. Cấu trúc giảm, nến nhấn chìm, vậy mà vài nến sau đã dính cắt lỗ, lý do nằm ở khung M15, đợt giảm đó nằm giữa vùng bò rất mạnh. Gấu con đang đánh vào căn cứ của bò mẹ. Trước khi tin tín hiệu, hãy hỏi 3 điều: Khung lớn có ngược mình không? Phe mình đã thất bại mấy lần ở đó? Và giá có đang đi ngang lộn xộn không? Nếu có, hãy đứng ngoài. Lỗi thứ hai: Vào lệnh ngược lại để gỡ. Vừa bị cắt lỗ là muốn gỡ ngay. Lệnh đó đến từ cảm xúc, không phải từ phương pháp. Nguy hiểm nhất là khi lệnh gỡ lại thắng. Bạn tưởng cách này hiệu quả, lần sau gấp đôi khối lượng. Một lệnh thắng chẳng chứng minh được gì. Lỗi thứ ba: Đóng lệnh vì giá lình xình. Vừa đóng ở hòa vốn thì giá chạy thẳng tới điểm chốt lời. Một lệnh thắng bị biến thành lệnh hòa/thua. Đã có phương pháp được kiểm chứng thì hãy tin nó, đúng quy tắc vào lệnh, đúng quy tắc chốt lời, không để cảm xúc chen vào. Tóm lại: Nhìn khung lớn trước, không vào lệnh để gỡ, không đóng lệnh trái quy tắc. Sửa được 3 lỗi này đáng giá hơn tìm một phương pháp mới. Theo dõi SO Trading để giao dịch kỷ luật hơn mỗi ngày.</t>
+          <t>ICT đã từng nói, tị trường chỉ làm có 2 việc thôi Thứ nhất là quay thanh khỏe và thứ 2 là lắp này các FVG Điều này có nghĩa là nếu như anh em vào một cái lệnh nào đó mà anh em chưa tìm nấy thanh khỏe thì rất có thể anh em sẽ trở thành thanh khỏe ICT là một trader với quan điểm dâu dịch là tị trường luôn luôn tìm thanh khỏe trước khi có những bước đi tiếp theo Thì sau khi tham khảo vào cái tư duy của ICT thì mình đã rút ra được một số các bài học và hôm nay mình sẽ chia sẻ anh em để có thể tăng thêm một cái tự lời hắn của mình Ok, nè Ma, thì anh em nhìn 2 cái bí vụ với đây thì anh em thấy khi giá nó phải hướng tới một cái buồn giá nào đó thì sẽ có 2 trường hợp xảy ra đúng không? Một là giá chạm đứng cái buồn này và tăng lên Nếu anh em ba này sẽ thắng Còn hai, nó chạm buồn này nhưng mà nó không tăng mà nó xuyên luôn thì anh em sẽ thua Anh em nghĩ là chỉ có 2 trường hợp thôi hả? Còn 1 trường hợp nữa đó là giá nó vét đáy xong nó mới thanh Đó Vậy thì nếu như anh em chọn 1 cái chờ về đây anh em ba lên thì anh em có tới 2 trường hợp mà anh em có thể thua được và là cái này và cái này Vậy thì thông bình hơn nó sẽ chờ cái gì? Ta sẽ chờ giá nó vét xong rồi chúng ta mới bầu lệnh thì lúc đó anh em có thể loại được bớt thêm 1 trường hợp thua nữa thì cái thể thắng nó sẽ tăng lên đúng không? Rồi bây giờ nó sẽ cùng nhau nhìn vào cái trạng này Đây là 1 cái cấu chút tăng đúng rồi anh em, chút tăng này thì có nhiều nên sẽ canh 3 cái giá qua bên bùn đáy này Thì khi giá trạm bùn đáy này nó sức hiểm cơ nến bin ba đứt rau thì là phần anh em sẽ vào buồn ở đây x lờ dưới cái đáy này và bề bề thì chúng ta cùng xem giá nó đi như thế nào hả? Mới vụng ta 1 vài trành bị x lờ sau đó nó mới tăng lên thì mình sẽ vào lệnh khi này bị béc rồi và tiếp tục tăng lên nè sau khi béc xong anh em phải tăng lên nó đóng đến qua cái nến này thì lúc này đây chỉ là 1 cái phá bởi giả thôi nè thì chúng ta mới bắt đầu vào lệnh mua vị trí này đạt sublots như đây và tb lên trần cùng xem giá nó chạy hả? Sau khi được bấy đựng sublots rồi thì giá nó đi rất là nhanh và đạt được tb đó là cách để thông minh nhớ nè chờ giá quá thân ngoại thông chúng ta mới vào chúng ta sẽ có tự lệnh hắn cao hơn ok nè mà lô video lại để xem kì cứng thiết</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1:21</t>
+          <t>1m - 11m</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696679708485897478</t>
+          <t>https://www.tiktok.com/@vn_rebates/video/7446381153868598534</t>
         </is>
       </c>
     </row>
@@ -2290,27 +2290,27 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Đọc nến theo luật bò gấu: vẽ căn cứ, chờ tín hiệu Đọc nến là đọc hành...</t>
+          <t>3 lỗi vào lệnh khiến bạn bị cắt lỗ oan (và cách sửa) Sửa lỗi quan trọ...</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Đọc nến theo luật bò gấu: vẽ căn cứ, chờ tín hiệu Đọc nến là đọc hành vi mua bán: phe nào chiếm ưu thế, phe nào cạn lực.</t>
+          <t>3 lỗi vào lệnh khiến bạn bị cắt lỗ oan (và cách sửa) Sửa lỗi quan trọng hơn tìm phương pháp mới. 3 lỗi hay gặp: tin tín hiệu khung nhỏ mà quên khung lớn, vào lệnh ngược để gỡ, đóng lệnh vì giá lình xình. Nguồn: nội dung do SO TRADING tự biên soạn. #Shorts #Trading</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Đọc nén không phải thuộc tên mẫu nén, mà là xem phê nào đang thắng. Trước hết, vẽ căn cứ của hai phê, vùng bò và vùng gấu ở khung đang giao dịch và khung kề trên. Giá chạy qua lại giữa hai vùng, có tín hiệu thì bật lại, không có thể phá qua vào vùng đổi vai. Vùng mạnh nhất là nơi bắt đầu một con sóng với những cây nén thân dài và giúp. Nhưng vùng mạnh mới là sắc xuất, cần thêm tín hiệu, nén nhỏ, dần có dâu hoặc cặp nén nhấn trìm. Tín hiệu xuất hiện lưng trừng thì kém tin cậy hơn tín hiệu ngay tại căn cứ. Tín hiệu đẹp mà tỉ lệ lời lộ kém hoặc ngực bối cảnh thì vẫn bỏ qua, phá thật hay phá giả. Xem nhịp hồi. Hồi về vùng vừa phá rồi đi tiếp theo hướng phá là phá thật, dữ lệnh bằng căn cứ. Rồi cắt lỗ ra sau căn cứ mới nhất và chốt khi ra tới căn cứ của phê kia. Bụng đích là sắc xuất cao, không phải thắng mọi lệnh. Tâm lý ổn định thì lợi nhuận mới đều. Theo dõi Sotrading để học đọc lên mỗi ngày.</t>
+          <t>Bị cắt lỗ oan liên tục, có thể lỗi nằm ở chính bạn, không phải phương pháp. Mới giao dịch, ai cũng đi tìm phương pháp tốt nhất. Nhưng sửa từng lỗi sai của mình còn quan trọng hơn nhiều. Lỗi thứ nhất: Thấy tín hiệu đẹp ở khung M5 mà quên nhìn khung lớn. Cấu trúc giảm, nến nhấn chìm, vậy mà vài nến sau đã dính cắt lỗ, lý do nằm ở khung M15, đợt giảm đó nằm giữa vùng bò rất mạnh. Gấu con đang đánh vào căn cứ của bò mẹ. Trước khi tin tín hiệu, hãy hỏi 3 điều: Khung lớn có ngược mình không? Phe mình đã thất bại mấy lần ở đó? Và giá có đang đi ngang lộn xộn không? Nếu có, hãy đứng ngoài. Lỗi thứ hai: Vào lệnh ngược lại để gỡ. Vừa bị cắt lỗ là muốn gỡ ngay. Lệnh đó đến từ cảm xúc, không phải từ phương pháp. Nguy hiểm nhất là khi lệnh gỡ lại thắng. Bạn tưởng cách này hiệu quả, lần sau gấp đôi khối lượng. Một lệnh thắng chẳng chứng minh được gì. Lỗi thứ ba: Đóng lệnh vì giá lình xình. Vừa đóng ở hòa vốn thì giá chạy thẳng tới điểm chốt lời. Một lệnh thắng bị biến thành lệnh hòa/thua. Đã có phương pháp được kiểm chứng thì hãy tin nó, đúng quy tắc vào lệnh, đúng quy tắc chốt lời, không để cảm xúc chen vào. Tóm lại: Nhìn khung lớn trước, không vào lệnh để gỡ, không đóng lệnh trái quy tắc. Sửa được 3 lỗi này đáng giá hơn tìm một phương pháp mới. Theo dõi SO Trading để giao dịch kỷ luật hơn mỗi ngày.</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>1:21</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696533638371970325</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696679708485897478</t>
         </is>
       </c>
     </row>
@@ -2340,27 +2340,27 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>7 bài học sau một buổi luyện tập giao dịch trên dữ liệu quá khứ #Shor...</t>
+          <t>Đọc nến theo luật bò gấu: vẽ căn cứ, chờ tín hiệu Đọc nến là đọc hành...</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>7 bài học sau một buổi luyện tập giao dịch trên dữ liệu quá khứ #Shorts Bảy bài học rút ra từ buổi luyện vào lệnh trên dữ liệu quá khứ BTCUSD (M15 + H1): bức tranh lớn, vùng cản, chờ tín hiệu, tỷ lệ lời/lỗ, lệnh chờ phá, quản lý lệnh và thống kê. Nguồn: nội dung do SO TRADING tự biên soạn. #Shorts #trading #bitcoin</t>
+          <t>Đọc nến theo luật bò gấu: vẽ căn cứ, chờ tín hiệu Đọc nến là đọc hành vi mua bán: phe nào chiếm ưu thế, phe nào cạn lực.</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Điện tập trên dữ liệu quá khứ, mình rút ra 7 bài học đáng giá 1. Xem bức tranh lớn trước. Khung lớn đi ngang thì đứng ngoài, hoặc chỉ canh vùng cản mạnh. 2. Chỉ vẽ vùng cản mạnh. Nơi bắt đầu còn sóng giúp. Vùng bị phá thì xóa đi. 3. Chờ phê ngực lại thất bại nhiều lần rồi mới vào. Đừng đặt sẵn lệnh trờ ngay vùng cản. 4. Tính tỉ lệ lời trên lỗ trước khi vào. Cản phía trước quá gần thì bỏ qua. 5. Dùng lệnh trờ phá để giá tự sắc nhận. Không phá thì lệnh không khớp, bạn không mất gì. 6. Rời cắt lỗ theo cấu trúc. Người mới cứ đặt chốt lời gấp đôi dùi do rồi để lệnh trại. 7. Đọc thống kê. Nhưng vài lệnh thì chưa nói lên điều gì. Cần hàng trăm lệnh mới đáng tin và chỉ luyện một phương pháp. Lặp lại đủ nhiều, nó sẽ thành phản xạ. Luyện tập không phải để đoán đúng từng lệnh, mà để đọc vùng cản, chờ tín hiệu và quản lý lệnh thành phản xạ. Theo dõi short reading để học thêm mỗi ngày.</t>
+          <t>Đọc nén không phải thuộc tên mẫu nén, mà là xem phê nào đang thắng. Trước hết, vẽ căn cứ của hai phê, vùng bò và vùng gấu ở khung đang giao dịch và khung kề trên. Giá chạy qua lại giữa hai vùng, có tín hiệu thì bật lại, không có thể phá qua vào vùng đổi vai. Vùng mạnh nhất là nơi bắt đầu một con sóng với những cây nén thân dài và giúp. Nhưng vùng mạnh mới là sắc xuất, cần thêm tín hiệu, nén nhỏ, dần có dâu hoặc cặp nén nhấn trìm. Tín hiệu xuất hiện lưng trừng thì kém tin cậy hơn tín hiệu ngay tại căn cứ. Tín hiệu đẹp mà tỉ lệ lời lộ kém hoặc ngực bối cảnh thì vẫn bỏ qua, phá thật hay phá giả. Xem nhịp hồi. Hồi về vùng vừa phá rồi đi tiếp theo hướng phá là phá thật, dữ lệnh bằng căn cứ. Rồi cắt lỗ ra sau căn cứ mới nhất và chốt khi ra tới căn cứ của phê kia. Bụng đích là sắc xuất cao, không phải thắng mọi lệnh. Tâm lý ổn định thì lợi nhuận mới đều. Theo dõi Sotrading để học đọc lên mỗi ngày.</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>55</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696421857871908116</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696533638371970325</t>
         </is>
       </c>
     </row>
@@ -2390,27 +2390,27 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Vào lệnh phá vỡ: 7 bài học chọn cú phá đẹp Không phải cú phá vỡ vùng ...</t>
+          <t>7 bài học sau một buổi luyện tập giao dịch trên dữ liệu quá khứ #Shor...</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Vào lệnh phá vỡ: 7 bài học chọn cú phá đẹp Không phải cú phá vỡ vùng cản nào cũng đáng vào lệnh. 7 bài học: vùng nhiều đỉnh, khung lớn, độ nén, chốt lời, dời cắt lỗ, ưu nhược điểm so với chờ hồi. Nguồn: nội dung do SO TRADING cung cấp. Nội dung chỉ mang tính giáo dục, không phải khuyến nghị đầu tư. #Shorts #trading #phavo</t>
+          <t>7 bài học sau một buổi luyện tập giao dịch trên dữ liệu quá khứ #Shorts Bảy bài học rút ra từ buổi luyện vào lệnh trên dữ liệu quá khứ BTCUSD (M15 + H1): bức tranh lớn, vùng cản, chờ tín hiệu, tỷ lệ lời/lỗ, lệnh chờ phá, quản lý lệnh và thống kê. Nguồn: nội dung do SO TRADING tự biên soạn. #Shorts #trading #bitcoin</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Không phải cú pha vỡ nào cũng đáng vào lệnh. Đây là 7 bài học để chọn cú pha đẹp. Giá phá qua vùng cản mới chỉ là điều kiện đầu tiên chưa đủ để vào lệnh. Phá vùng nhiều đỉnh mạnh hơn phá một đỉnh vì phê bán đã rồn hết lực mà vẫn thua. Nhìn khung lớn hơn để biết phê mua có chiếm yêu thế. Và lệnh có thể đi xa tới đầu. Đẹp nhất là khi các đáy cao dần nén sát vùng đỉnh rồi bung lên. Cắt lỗ đặt dưới đáy gần nhất. Đặt trốt lời gấp đôi rủi do rồi nhìn sang bên trái. Có vùng cản nguy hiểm phía trước thì bỏ qua. Giá đi đúng hướng thì dời điểm cắt lỗ lên dưới đáy cao hơn mới. Lệnh phá vỡ cho kết quả rất nhanh vì phê ngược lại đã cạn lực. Nhưng chọn điểm vào kém thì cắt lỗ rất xa. Làm hỏng tỷ lệ lời trên lỗ. Chờ giá hồi về thì cắt lỗ ngắn hơn nhưng giá thường phải đi ngang một thời gian. Tìm vùng nhiều đỉnh, chờ giá nén rồi phá và chỉ vào khi phía trước còn chỗ chạy. Theo dõi SO Trading để xem thêm.</t>
+          <t>Điện tập trên dữ liệu quá khứ, mình rút ra 7 bài học đáng giá 1. Xem bức tranh lớn trước. Khung lớn đi ngang thì đứng ngoài, hoặc chỉ canh vùng cản mạnh. 2. Chỉ vẽ vùng cản mạnh. Nơi bắt đầu còn sóng giúp. Vùng bị phá thì xóa đi. 3. Chờ phê ngực lại thất bại nhiều lần rồi mới vào. Đừng đặt sẵn lệnh trờ ngay vùng cản. 4. Tính tỉ lệ lời trên lỗ trước khi vào. Cản phía trước quá gần thì bỏ qua. 5. Dùng lệnh trờ phá để giá tự sắc nhận. Không phá thì lệnh không khớp, bạn không mất gì. 6. Rời cắt lỗ theo cấu trúc. Người mới cứ đặt chốt lời gấp đôi dùi do rồi để lệnh trại. 7. Đọc thống kê. Nhưng vài lệnh thì chưa nói lên điều gì. Cần hàng trăm lệnh mới đáng tin và chỉ luyện một phương pháp. Lặp lại đủ nhiều, nó sẽ thành phản xạ. Luyện tập không phải để đoán đúng từng lệnh, mà để đọc vùng cản, chờ tín hiệu và quản lý lệnh thành phản xạ. Theo dõi short reading để học thêm mỗi ngày.</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>54</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696331802654280980</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696421857871908116</t>
         </is>
       </c>
     </row>
@@ -2440,27 +2440,27 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Giao dịch như lính bắn tỉa: đo độ chính xác, đừng đếm số lệnh 7 bài h...</t>
+          <t>Vào lệnh phá vỡ: 7 bài học chọn cú phá đẹp Không phải cú phá vỡ vùng ...</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Giao dịch như lính bắn tỉa: đo độ chính xác, đừng đếm số lệnh 7 bài học từ hình ảnh lính bắn tỉa: chính xác hơn số lượng, kẻ thù là chính mình, phương pháp là vũ khí, luyện hàng nghìn lần, luyện trên dữ liệu quá khứ, tự bóp cò, khung nhỏ không nhiễu. Nguồn: nội dung do kênh SO TRADING tổng hợp. Chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #giaodich #trading</t>
+          <t>Vào lệnh phá vỡ: 7 bài học chọn cú phá đẹp Không phải cú phá vỡ vùng cản nào cũng đáng vào lệnh. 7 bài học: vùng nhiều đỉnh, khung lớn, độ nén, chốt lời, dời cắt lỗ, ưu nhược điểm so với chờ hồi. Nguồn: nội dung do SO TRADING cung cấp. Nội dung chỉ mang tính giáo dục, không phải khuyến nghị đầu tư. #Shorts #trading #phavo</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>Lính bán tỉa, không bán ít. Họ bán chính xác, bán tỉa là độ chính xác, không phải ít hay nhiều lệnh. Vào ít mà sai nhiều thì vẫn không giỏi, kẻ thù không phải thị trường. Bạn không điều khiển được giá, chỉ điều khiển được chính mình. Phương Pháp là vũ khí. Đừng ra chận tay không, cũng đừng mang quá nhiều thứ mà không thạo thứ nào. Sạ thủ giỏi bán hàng nghìn viên khi luyện tập. Simo hay he hạ khoảng 500 linh năm mục tiêu trong 100 ngày. Các luyện nhanh nhất là vào lệnh trên dữ liệu quá khứ. Một giờ tua biểu đồ bằng 6 tuần giao dịch thật. Càng nhiều lệnh, bạn càng sớm thấy lỗi của mình, mà không tốn một đồng tiền thật. Gia trận thì tự mình bóp cỏ. Theo tín hiệu mù quán, không ai có lợi nhuận ổn địch. Không nhỏ, không hề nhéo, chỉ là bạn chưa hiểu. Luyện đủ lâu, biểu đồ nào cũng đọc được. Đừng đếm số lệnh, hãy đò độ chính xác của mỗi phát bán theo dõi Soul Trading để luyện từng phát bán chính xác hơn.</t>
+          <t>Không phải cú pha vỡ nào cũng đáng vào lệnh. Đây là 7 bài học để chọn cú pha đẹp. Giá phá qua vùng cản mới chỉ là điều kiện đầu tiên chưa đủ để vào lệnh. Phá vùng nhiều đỉnh mạnh hơn phá một đỉnh vì phê bán đã rồn hết lực mà vẫn thua. Nhìn khung lớn hơn để biết phê mua có chiếm yêu thế. Và lệnh có thể đi xa tới đầu. Đẹp nhất là khi các đáy cao dần nén sát vùng đỉnh rồi bung lên. Cắt lỗ đặt dưới đáy gần nhất. Đặt trốt lời gấp đôi rủi do rồi nhìn sang bên trái. Có vùng cản nguy hiểm phía trước thì bỏ qua. Giá đi đúng hướng thì dời điểm cắt lỗ lên dưới đáy cao hơn mới. Lệnh phá vỡ cho kết quả rất nhanh vì phê ngược lại đã cạn lực. Nhưng chọn điểm vào kém thì cắt lỗ rất xa. Làm hỏng tỷ lệ lời trên lỗ. Chờ giá hồi về thì cắt lỗ ngắn hơn nhưng giá thường phải đi ngang một thời gian. Tìm vùng nhiều đỉnh, chờ giá nén rồi phá và chỉ vào khi phía trước còn chỗ chạy. Theo dõi SO Trading để xem thêm.</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>54</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696144076411817268</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696331802654280980</t>
         </is>
       </c>
     </row>
@@ -2490,27 +2490,27 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Kế hoạch một ngày giao dịch: 7 bài học để không chơi cho vui Giao dịc...</t>
+          <t>Giao dịch như lính bắn tỉa: đo độ chính xác, đừng đếm số lệnh 7 bài h...</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Kế hoạch một ngày giao dịch: 7 bài học để không chơi cho vui Giao dịch thành công không cao siêu, nó dành cho người có kế hoạch. 7 bài học: coi giao dịch là công việc, chọn khung giờ cố định, lướt nhanh đầu ngày, đừng ép vào lệnh, luyện tập thật nhiều, không dán mắt vào giá, kiểm tra trước khi vào lệnh. Nguồn: nội dung do kênh SO TRADING tổng hợp. Nội dung chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #giaodich #trading #kehoach</t>
+          <t>Giao dịch như lính bắn tỉa: đo độ chính xác, đừng đếm số lệnh 7 bài học từ hình ảnh lính bắn tỉa: chính xác hơn số lượng, kẻ thù là chính mình, phương pháp là vũ khí, luyện hàng nghìn lần, luyện trên dữ liệu quá khứ, tự bóp cò, khung nhỏ không nhiễu. Nguồn: nội dung do kênh SO TRADING tổng hợp. Chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #giaodich #trading</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Giao dịch như một trò chơi, đó là cách nhanh nhất để mất tiền, hãy coi giao dịch là công việc. Tự do, nhưng phải có kế hoạch rõ ràng, chọn một khung giờ cố định trùng lúc thị trường mạnh nhất, phiên Âu và phiên Mỹ không cần ngồi cả ngày. Não không thể tập trung liên tục, nhất là khi có tiền dính vào, đầu ngày, lượt nhanh các cặp tiền khoảng 10 phút để nắm su hướng, rồi tắt máy, đừng cố tìm lý do để vào lệnh. Không giao dịch cũng là một phần của công việc. Phần lớn thời gian là luyện tập, 99 phần chuẩn bị, một phần thực chiến để biểu đồ sắn nhưng đừng dám mắt vào giá. Liết trưa đầy một phút là đủ, trước khi vào lệnh, kiểm tra, su hướng lớn, vùng cản, điểm cắt lỗ và tỷ lệ lời trên lỗ, vào lệnh rồi thì đừng ngồi canh và đừng kỳ vọng thắng mọi lệnh vài lệnh không nói lên điều gì. Kết quả chỉ rõ khi số lệnh đủ nhiều, ưu khóa cần nhớ là chuẩn bị. Theo dõi show trading để xây kế hoạch giao dịch của riêng bạn.</t>
+          <t>Lính bán tỉa, không bán ít. Họ bán chính xác, bán tỉa là độ chính xác, không phải ít hay nhiều lệnh. Vào ít mà sai nhiều thì vẫn không giỏi, kẻ thù không phải thị trường. Bạn không điều khiển được giá, chỉ điều khiển được chính mình. Phương Pháp là vũ khí. Đừng ra chận tay không, cũng đừng mang quá nhiều thứ mà không thạo thứ nào. Sạ thủ giỏi bán hàng nghìn viên khi luyện tập. Simo hay he hạ khoảng 500 linh năm mục tiêu trong 100 ngày. Các luyện nhanh nhất là vào lệnh trên dữ liệu quá khứ. Một giờ tua biểu đồ bằng 6 tuần giao dịch thật. Càng nhiều lệnh, bạn càng sớm thấy lỗi của mình, mà không tốn một đồng tiền thật. Gia trận thì tự mình bóp cỏ. Theo tín hiệu mù quán, không ai có lợi nhuận ổn địch. Không nhỏ, không hề nhéo, chỉ là bạn chưa hiểu. Luyện đủ lâu, biểu đồ nào cũng đọc được. Đừng đếm số lệnh, hãy đò độ chính xác của mỗi phát bán theo dõi Soul Trading để luyện từng phát bán chính xác hơn.</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>55</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7696052072612973844</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696144076411817268</t>
         </is>
       </c>
     </row>
@@ -2540,27 +2540,27 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>Độ nén của giá: 7 điều giúp cắt lỗ ngắn, thắng nhiều hơn #Shorts Độ n...</t>
+          <t>Kế hoạch một ngày giao dịch: 7 bài học để không chơi cho vui Giao dịc...</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Độ nén của giá: 7 điều giúp cắt lỗ ngắn, thắng nhiều hơn #Shorts Độ nén của giá là gì, vì sao giá nén rồi bung, cách nhìn hình dạng vùng nén và đặt cắt lỗ ngắn mà an toàn. Nội dung do kênh SO TRADING tổng hợp. Giao dịch luôn có rủi ro, đây không phải lời khuyên đầu tư. #Shorts #trading #giaodich</t>
+          <t>Kế hoạch một ngày giao dịch: 7 bài học để không chơi cho vui Giao dịch thành công không cao siêu, nó dành cho người có kế hoạch. 7 bài học: coi giao dịch là công việc, chọn khung giờ cố định, lướt nhanh đầu ngày, đừng ép vào lệnh, luyện tập thật nhiều, không dán mắt vào giá, kiểm tra trước khi vào lệnh. Nguồn: nội dung do kênh SO TRADING tổng hợp. Nội dung chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #giaodich #trading #kehoach</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Có một điều ít ai nói tới, nhưng giúp bạn thắng nhiều hơn và cắt lỗ ngắn hơn, đó là độ nén của giá. Hôm nay mình đi qua 7 điều cần nắm. 1. Giá đi ngang, đáy cao dần, đỉnh thấp dần, biên độ thu hẹp, tức là giá đăng nén. Nén càng sát nhau thì nén càng mạnh, sống bên trong càng lớn thì nén càng yếu. 2. Giá nén vì lực 2 phê ngang nhau, phê mua đẩy đáy lên, phê bán ép đỉnh xuống. 3. Nén thì sẽ bung như quả bóng bơm quá căng, nén càng mạnh, bung càng mạnh. Hướng bung thì nhìn bối cảnh lớn, trong xu hướng tăng dễ phá lên, trong vùng giảm dễ phá xuống. 4. Tất cả chỉ là sắc suất, việc của mình là tăng sắc suất, không tìm sự chắc chắn. 5. Tạm ra cần là hai phê ngang sức, đáy giúp lên là phê mua mạnh hơn, đỉnh giúp xuống là phê bán mạnh hơn, vùng giá mở rộng như cái loa thì đứng ngoài. Vì cả hai phê đều loạn. 6. Vùng nén cho điểm cắt lỗ vừa an toàn vừa ngắn vì vào lệnh ngay chỗ giá hẹp nhất. 7. Đừng rời cắt lỗ ra xa. Giá đã phá căn cứ thì phê kia đã thắng thế, tìm vùng nén, chờ giá bùng, vào lệnh với cắt lỗ ngắn. Theo dõi show trading để học thêm.</t>
+          <t>Giao dịch như một trò chơi, đó là cách nhanh nhất để mất tiền, hãy coi giao dịch là công việc. Tự do, nhưng phải có kế hoạch rõ ràng, chọn một khung giờ cố định trùng lúc thị trường mạnh nhất, phiên Âu và phiên Mỹ không cần ngồi cả ngày. Não không thể tập trung liên tục, nhất là khi có tiền dính vào, đầu ngày, lượt nhanh các cặp tiền khoảng 10 phút để nắm su hướng, rồi tắt máy, đừng cố tìm lý do để vào lệnh. Không giao dịch cũng là một phần của công việc. Phần lớn thời gian là luyện tập, 99 phần chuẩn bị, một phần thực chiến để biểu đồ sắn nhưng đừng dám mắt vào giá. Liết trưa đầy một phút là đủ, trước khi vào lệnh, kiểm tra, su hướng lớn, vùng cản, điểm cắt lỗ và tỷ lệ lời trên lỗ, vào lệnh rồi thì đừng ngồi canh và đừng kỳ vọng thắng mọi lệnh vài lệnh không nói lên điều gì. Kết quả chỉ rõ khi số lệnh đủ nhiều, ưu khóa cần nhớ là chuẩn bị. Theo dõi show trading để xây kế hoạch giao dịch của riêng bạn.</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1:10</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695960796676803861</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7696052072612973844</t>
         </is>
       </c>
     </row>
@@ -2590,27 +2590,27 @@
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Hiểu đúng đa khung thời gian: 6 điều đừng học vẹt Sáu điều cần hiểu đ...</t>
+          <t>Độ nén của giá: 7 điều giúp cắt lỗ ngắn, thắng nhiều hơn #Shorts Độ n...</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Hiểu đúng đa khung thời gian: 6 điều đừng học vẹt Sáu điều cần hiểu đúng về đa khung thời gian trong giao dịch: không cần xem nhiều khung, không cần cùng hướng, vùng cản lớn nhỏ và cách vào lệnh theo cung cầu. #Shorts #trading #dakhungthoigian</t>
+          <t>Độ nén của giá: 7 điều giúp cắt lỗ ngắn, thắng nhiều hơn #Shorts Độ nén của giá là gì, vì sao giá nén rồi bung, cách nhìn hình dạng vùng nén và đặt cắt lỗ ngắn mà an toàn. Nội dung do kênh SO TRADING tổng hợp. Giao dịch luôn có rủi ro, đây không phải lời khuyên đầu tư. #Shorts #trading #giaodich</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Xem nhiều khung thời gian hơn, không có nghĩa là giao dịch tốt hơn. Đa khung thời gian, ai cũng quan tâm, nhưng nhiều người chỉ học vẹt. Đây là 6 điều cần hiểu đúng. 1. Xem nhiều khung, không phải càng nhiều càng tốt. Lệnh ở khung 10 năm, chỉ 5 trong 1, 2 cây đến hức 4, còn chưa hết 1 đến ngày. Cùng quá lớn gần như không có tác dụng với lệnh đó. Xem chúng chỉ làm bạn phân vần khi tín hiệu đẹp xuất hiện. 2. Không cần mọi khung cùng 1 hướng. Khung lớn có thể đang giảm, nhưng 1 cây nén tăng của nó là cả su hướng tăng dài ở khung nhỏ. 3. Khung thời gian, chỉ là cách con người đóng khung giá. Giá đi thành 1 đường duy nhất như sợi chỉ, gom lại thì thành nén. 4. Không có vùng cản của 15 hay của 1. Chỉ có vùng cản lớn hơn và vùng cản nhỏ hơn. 5. Muốn nhìn tổng thể, hãy thu nhỏ biểu đồ hoặc lên đúng 1 khung kỳ trên. Đừng nhảy lên khung quá xa. 6. Vào lệnh theo kịch bản cung cầu. Giá phá đỉnh cũ rồi đi ngang, phê mua chiếm ưu thế thì chờ giá phá vùng đỉnh đó. Khi đó vào lệnh mua, cách lỗ đặt dưới vùng vừa phá chất lời nhắm tới vùng cản lớn hơn phía trên. Đừng học thuộc phải xem bao nhiêu khung. Hãy hiểu giá được tạo ra thế nào, rồi chọn cách nhìn thuận tiện nhất cho mình. Rưu duy sai giống con đỉa, bám càng lâu càng hút cạn tiền bạc. Theo dõi sò trading để giao dịch đúng bản chất.</t>
+          <t>Có một điều ít ai nói tới, nhưng giúp bạn thắng nhiều hơn và cắt lỗ ngắn hơn, đó là độ nén của giá. Hôm nay mình đi qua 7 điều cần nắm. 1. Giá đi ngang, đáy cao dần, đỉnh thấp dần, biên độ thu hẹp, tức là giá đăng nén. Nén càng sát nhau thì nén càng mạnh, sống bên trong càng lớn thì nén càng yếu. 2. Giá nén vì lực 2 phê ngang nhau, phê mua đẩy đáy lên, phê bán ép đỉnh xuống. 3. Nén thì sẽ bung như quả bóng bơm quá căng, nén càng mạnh, bung càng mạnh. Hướng bung thì nhìn bối cảnh lớn, trong xu hướng tăng dễ phá lên, trong vùng giảm dễ phá xuống. 4. Tất cả chỉ là sắc suất, việc của mình là tăng sắc suất, không tìm sự chắc chắn. 5. Tạm ra cần là hai phê ngang sức, đáy giúp lên là phê mua mạnh hơn, đỉnh giúp xuống là phê bán mạnh hơn, vùng giá mở rộng như cái loa thì đứng ngoài. Vì cả hai phê đều loạn. 6. Vùng nén cho điểm cắt lỗ vừa an toàn vừa ngắn vì vào lệnh ngay chỗ giá hẹp nhất. 7. Đừng rời cắt lỗ ra xa. Giá đã phá căn cứ thì phê kia đã thắng thế, tìm vùng nén, chờ giá bùng, vào lệnh với cắt lỗ ngắn. Theo dõi show trading để học thêm.</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1:19</t>
+          <t>1:10</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695799603068734741</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695960796676803861</t>
         </is>
       </c>
     </row>
@@ -2640,27 +2640,27 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>7 bài học sau 5 năm đi cùng thị trường | SO TRADING Bảy bài học kinh ...</t>
+          <t>Hiểu đúng đa khung thời gian: 6 điều đừng học vẹt Sáu điều cần hiểu đ...</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>7 bài học sau 5 năm đi cùng thị trường | SO TRADING Bảy bài học kinh nghiệm sau 5 năm tham gia thị trường: biết đứng ngoài, có kịch bản, quản lý rủi ro, tránh khoảng trống cuối tuần. #trading #crypto #fx</t>
+          <t>Hiểu đúng đa khung thời gian: 6 điều đừng học vẹt Sáu điều cần hiểu đúng về đa khung thời gian trong giao dịch: không cần xem nhiều khung, không cần cùng hướng, vùng cản lớn nhỏ và cách vào lệnh theo cung cầu. #Shorts #trading #dakhungthoigian</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>SU Trading chia sẻ 5 năm trong thị trường mình rút ra 7 bài học này 1. Thị trường đi ngang thì đứng ngoài chỉ hành động khi khung lớn cho lý do rõ ràng 2. Có kịch bản trước khi vào lệnh Giá không phá nổi vùng cản thì thoát dù lời chưa nhiều 3. Điểm vào chưa đẹp thì chờ ở vùng tốt hơn để cắt lỗ gần hơn và rủi do nhỏ hơn 4. Lệnh đang lời thì rời cắt lỗ về hòa vốn và chốt trước 1 phần khi giá chạm vùng nguy hiểm 5. Đừng giữ lệnh ngắn hạn qua cuối tuần vì khoảng chống giá đầu tuần rất nguy hiểm 6. Đừng bắt đầu bằng khung thời gian nhỏ Chọn khung lớn đặt lệnh xong rồi để đó 7. Ýt yếu tố ủng hộ thì khả năng thắng thấp Và thua như vậy là bình thường, muốn biết phương pháp hiệu quả đến đâu Hãy thống kê theo từng cặp tiền và từng khung thời gian Tóm lại, đứng ngoài khi thị trường không rõ và luôn có kịch bản trước khi vào lệnh Đây là kinh nghiệm cá nhân, không phải lời khuyên đầu tư Gé SO Trading để cùng trao đổi thêm nhé!</t>
+          <t>Xem nhiều khung thời gian hơn, không có nghĩa là giao dịch tốt hơn. Đa khung thời gian, ai cũng quan tâm, nhưng nhiều người chỉ học vẹt. Đây là 6 điều cần hiểu đúng. 1. Xem nhiều khung, không phải càng nhiều càng tốt. Lệnh ở khung 10 năm, chỉ 5 trong 1, 2 cây đến hức 4, còn chưa hết 1 đến ngày. Cùng quá lớn gần như không có tác dụng với lệnh đó. Xem chúng chỉ làm bạn phân vần khi tín hiệu đẹp xuất hiện. 2. Không cần mọi khung cùng 1 hướng. Khung lớn có thể đang giảm, nhưng 1 cây nén tăng của nó là cả su hướng tăng dài ở khung nhỏ. 3. Khung thời gian, chỉ là cách con người đóng khung giá. Giá đi thành 1 đường duy nhất như sợi chỉ, gom lại thì thành nén. 4. Không có vùng cản của 15 hay của 1. Chỉ có vùng cản lớn hơn và vùng cản nhỏ hơn. 5. Muốn nhìn tổng thể, hãy thu nhỏ biểu đồ hoặc lên đúng 1 khung kỳ trên. Đừng nhảy lên khung quá xa. 6. Vào lệnh theo kịch bản cung cầu. Giá phá đỉnh cũ rồi đi ngang, phê mua chiếm ưu thế thì chờ giá phá vùng đỉnh đó. Khi đó vào lệnh mua, cách lỗ đặt dưới vùng vừa phá chất lời nhắm tới vùng cản lớn hơn phía trên. Đừng học thuộc phải xem bao nhiêu khung. Hãy hiểu giá được tạo ra thế nào, rồi chọn cách nhìn thuận tiện nhất cho mình. Rưu duy sai giống con đỉa, bám càng lâu càng hút cạn tiền bạc. Theo dõi sò trading để giao dịch đúng bản chất.</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>1:19</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695696836140616980</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695799603068734741</t>
         </is>
       </c>
     </row>
@@ -2690,27 +2690,27 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>7 bài học từ 3 lệnh thực tế: 2 thắng, 1 thua vì lỗi bất cẩn Hai lệnh ...</t>
+          <t>7 bài học sau 5 năm đi cùng thị trường | SO TRADING Bảy bài học kinh ...</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>7 bài học từ 3 lệnh thực tế: 2 thắng, 1 thua vì lỗi bất cẩn Hai lệnh thắng, một lệnh thua vì một lỗi bất cẩn. Bảy bài học về chờ xu hướng rõ, vào lệnh khi đủ yếu tố, đặt lệnh chờ, quản lý khối lượng, kiểm soát cảm xúc và giữ điểm cắt lỗ. Nguồn: kinh nghiệm giao dịch thực tế của SO TRADING. #Shorts #trading #giaodich</t>
+          <t>7 bài học sau 5 năm đi cùng thị trường | SO TRADING Bảy bài học kinh nghiệm sau 5 năm tham gia thị trường: biết đứng ngoài, có kịch bản, quản lý rủi ro, tránh khoảng trống cuối tuần. #trading #crypto #fx</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>2 lệnh thắng, 1 lệnh thua vì 1 lỗi bất cảnh. Đây là 7 bài học đắt giá. 1. Su hướng gió là lợi thế lớn nhất. Nó không xuất hiện thường xuyên nên hãy kiên nhận trở. 2. Gom đủ 3 yếu tố rồi mới vào. Su hướng vung cản của phê mình và tín hiệu đến xác nhận. 3. Giá đã chạy xa thì đặt lệnh trở vùng đỉnh cũ. Không khớp cũng không mất tiền, tính khối lượng trước để biết thua mất bao nhiêu. Chốt lời mặc định gấp 2 lần rủi do. 4. Tận dụng núp phê nâu mở cửa, đầu giờ chiều giờ Việt Nam khi tín hiệu xuất hiện nhiều. 5. Vào lệnh xong đừng nhìn biểu đồ quá nhiều, nhìn nhiều dễ chốt sớm rồi tiếc, hãy gạt cảm xúc gắn với tiền. Chỉ vui khi làm đúng kịch bản, chỉ ái náy khi làm sai kịch bản. 6. Lệnh rủi do thì hoặc đứng ngoài, hoặc canh tới nơi tới chốn. Không canh được thì đóng lệnh. 7. Giữ điểm cắt lỗ, đừng rời hay bỏ, và xem lại lệnh cũ để thấy lỗi hay lặp lại. Còn vốn thì còn lấy lại được, và phần lời chính là kinh nghiệm, trở xu hướng rõ, đủ yếu tố mới vào, làm đúng kịch bản. Theo dõi SO Trading để học giao dịch có kỷ luật.</t>
+          <t>SU Trading chia sẻ 5 năm trong thị trường mình rút ra 7 bài học này 1. Thị trường đi ngang thì đứng ngoài chỉ hành động khi khung lớn cho lý do rõ ràng 2. Có kịch bản trước khi vào lệnh Giá không phá nổi vùng cản thì thoát dù lời chưa nhiều 3. Điểm vào chưa đẹp thì chờ ở vùng tốt hơn để cắt lỗ gần hơn và rủi do nhỏ hơn 4. Lệnh đang lời thì rời cắt lỗ về hòa vốn và chốt trước 1 phần khi giá chạm vùng nguy hiểm 5. Đừng giữ lệnh ngắn hạn qua cuối tuần vì khoảng chống giá đầu tuần rất nguy hiểm 6. Đừng bắt đầu bằng khung thời gian nhỏ Chọn khung lớn đặt lệnh xong rồi để đó 7. Ýt yếu tố ủng hộ thì khả năng thắng thấp Và thua như vậy là bình thường, muốn biết phương pháp hiệu quả đến đâu Hãy thống kê theo từng cặp tiền và từng khung thời gian Tóm lại, đứng ngoài khi thị trường không rõ và luôn có kịch bản trước khi vào lệnh Đây là kinh nghiệm cá nhân, không phải lời khuyên đầu tư Gé SO Trading để cùng trao đổi thêm nhé!</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1:09</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695602506377809173</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695696836140616980</t>
         </is>
       </c>
     </row>
@@ -2740,27 +2740,27 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>3 lỗi tâm lý giao dịch khiến bạn cháy tài khoản (và cách sửa) Phương ...</t>
+          <t>7 bài học từ 3 lệnh thực tế: 2 thắng, 1 thua vì lỗi bất cẩn Hai lệnh ...</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
         <is>
-          <t>3 lỗi tâm lý giao dịch khiến bạn cháy tài khoản (và cách sửa) Phương pháp chỉ là một phần, tâm lý mới quyết định. 3 lỗi gần như ai cũng gặp: sợ bỏ lỡ (FOMO), trả thù thị trường, chốt lời sớm - gồng lỗ dài, cùng cách sửa đơn giản cho từng lỗi. Nguồn: nội dung BlackRose Admin (08/10/2026), biên soạn lại bởi SO TRADING. Nội dung chỉ mang tính tham khảo, không phải khuyến nghị đầu tư. #Shorts #trading #tamlygiaodich</t>
+          <t>7 bài học từ 3 lệnh thực tế: 2 thắng, 1 thua vì lỗi bất cẩn Hai lệnh thắng, một lệnh thua vì một lỗi bất cẩn. Bảy bài học về chờ xu hướng rõ, vào lệnh khi đủ yếu tố, đặt lệnh chờ, quản lý khối lượng, kiểm soát cảm xúc và giữ điểm cắt lỗ. Nguồn: kinh nghiệm giao dịch thực tế của SO TRADING. #Shorts #trading #giaodich</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Ba lỗi tâm lý này đang âm thầm đốt tài khoản của bạn. Phương pháp giao dịch không phải tất cả. Phần lớn thành công đến từ tâm lý. Lỗi 1. Sợ bỏ lỡ cơ hội. Thấy giá chạy, thấy người khác lời là vào lệnh bừa. Cách sửa, rời nhóm chát tín hiệu, tự luyện tập và xây chiến lược vào lệnh của riêng bạn. Lỗi 2. Chả thủ tị trường. Thua xong là gấp đôi khối lượng để gỡ lại. Cách sửa. Chỉ nắp ít khoảng 2 phần chăm vốn để có khoảng dừng mà tỉnh lại và đi từ nhỏ đến lớn. 10 đô và 1 nghìn đô cho cảm xúc rất khác nhau. Lỗi 3. Chốt lời sớm, gồng lỗ dài. Thắng thì ăn ít, thua thì lỗ nhiều. Cách sửa. Đặt sẵn chốt lời và cắt lỗ. Ban đầu cho 2 mức bằng nhau. Đặt xong thì đừng nhìn tài khoản. Giữ từ 1 tuần đến 1 tháng để thành thói quen. Ba lỗi như 3 tảng đá trên đường. Quay lại. Hoặc vượt qua từng tảng 1. Bạn đang vướng lỗi nào? Theo dõi sốt trading để học giao dịch bên vững hơn.</t>
+          <t>2 lệnh thắng, 1 lệnh thua vì 1 lỗi bất cảnh. Đây là 7 bài học đắt giá. 1. Su hướng gió là lợi thế lớn nhất. Nó không xuất hiện thường xuyên nên hãy kiên nhận trở. 2. Gom đủ 3 yếu tố rồi mới vào. Su hướng vung cản của phê mình và tín hiệu đến xác nhận. 3. Giá đã chạy xa thì đặt lệnh trở vùng đỉnh cũ. Không khớp cũng không mất tiền, tính khối lượng trước để biết thua mất bao nhiêu. Chốt lời mặc định gấp 2 lần rủi do. 4. Tận dụng núp phê nâu mở cửa, đầu giờ chiều giờ Việt Nam khi tín hiệu xuất hiện nhiều. 5. Vào lệnh xong đừng nhìn biểu đồ quá nhiều, nhìn nhiều dễ chốt sớm rồi tiếc, hãy gạt cảm xúc gắn với tiền. Chỉ vui khi làm đúng kịch bản, chỉ ái náy khi làm sai kịch bản. 6. Lệnh rủi do thì hoặc đứng ngoài, hoặc canh tới nơi tới chốn. Không canh được thì đóng lệnh. 7. Giữ điểm cắt lỗ, đừng rời hay bỏ, và xem lại lệnh cũ để thấy lỗi hay lặp lại. Còn vốn thì còn lấy lại được, và phần lời chính là kinh nghiệm, trở xu hướng rõ, đủ yếu tố mới vào, làm đúng kịch bản. Theo dõi SO Trading để học giao dịch có kỷ luật.</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>1:09</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695389393443409173</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695602506377809173</t>
         </is>
       </c>
     </row>
@@ -2790,27 +2790,27 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Chứng khoán, tiền điện tử hay ngoại hối: chọn thị trường nào? So sánh...</t>
+          <t>3 lỗi tâm lý giao dịch khiến bạn cháy tài khoản (và cách sửa) Phương ...</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Chứng khoán, tiền điện tử hay ngoại hối: chọn thị trường nào? So sánh 3 thị trường theo 4 đặc điểm: pháp lý, thanh khoản, thời gian giao dịch, nền tảng. Nguồn: nội dung do tác giả cung cấp. #Shorts #trading #xuhuong #crypto #fx</t>
+          <t>3 lỗi tâm lý giao dịch khiến bạn cháy tài khoản (và cách sửa) Phương pháp chỉ là một phần, tâm lý mới quyết định. 3 lỗi gần như ai cũng gặp: sợ bỏ lỡ (FOMO), trả thù thị trường, chốt lời sớm - gồng lỗ dài, cùng cách sửa đơn giản cho từng lỗi. Nguồn: nội dung BlackRose Admin (08/10/2026), biên soạn lại bởi SO TRADING. Nội dung chỉ mang tính tham khảo, không phải khuyến nghị đầu tư. #Shorts #trading #tamlygiaodich</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Trứng khoán, tiền điện tử hay ngoại hối, chọn sai thị trường là mất tiền. Bối thị trường có đặc điểm riêng, hãy xét bốn thứ, pháp lý, thanh khoản, thời gian giao dịch và nền tảng. Pháp lý, trứng khoán được nhà nước bảo hộ chặt trẽ. Tiền điện tử và ngoại hối thì chưa được công nhận. Vì vậy, giữ số tiền lớn lâu dài thì trứng khoán an toàn hơn, đừng ném cả tài sản vào sản không tên tuổi. Thanh khoản, ngoại hối lớn nhất, rồi trứng khoán, rồi tiền điện tử. Nhưng trứng khoán Việt Nam thấp nhất nên chỉ hợp đầu tư dài hạn. Cổ phiếu và tiền điện tử dễ bị thao túng, biến động vài chục phần trăm. Cặp tiền lệch 1 phần trăm 1 ngày đã là nhiều. Thời gian, trứng khoán chỉ mở khoảng 4 tiếng 1 ngày, ngoại hối 24h, 5 ngày, tiền điện tử 24h, 7 ngày, nền tảng. Sanh ngoại hối giao dịch được tiền tệ, tiền điện tử, chỉ số và vàng. Nhưng đó là hợp đồng tranh lệch bạn không sở hữu tài sản. Tóm lại, trứng khoán hợp dài hạn, ngoại hối chỉ hợp ngắn hạn. Tiền điện tử hợp cả 2 nhưng rủi do cao, và dù chọn thị trường nào cũng phải chọn sản uy tín. Sanh kém thì ở đâu cũng dễ mất tiền, theo dõi để học cách bảo vệ và làm sinh lời đồng vốn của bạn mỗi ngày.</t>
+          <t>Ba lỗi tâm lý này đang âm thầm đốt tài khoản của bạn. Phương pháp giao dịch không phải tất cả. Phần lớn thành công đến từ tâm lý. Lỗi 1. Sợ bỏ lỡ cơ hội. Thấy giá chạy, thấy người khác lời là vào lệnh bừa. Cách sửa, rời nhóm chát tín hiệu, tự luyện tập và xây chiến lược vào lệnh của riêng bạn. Lỗi 2. Chả thủ tị trường. Thua xong là gấp đôi khối lượng để gỡ lại. Cách sửa. Chỉ nắp ít khoảng 2 phần chăm vốn để có khoảng dừng mà tỉnh lại và đi từ nhỏ đến lớn. 10 đô và 1 nghìn đô cho cảm xúc rất khác nhau. Lỗi 3. Chốt lời sớm, gồng lỗ dài. Thắng thì ăn ít, thua thì lỗ nhiều. Cách sửa. Đặt sẵn chốt lời và cắt lỗ. Ban đầu cho 2 mức bằng nhau. Đặt xong thì đừng nhìn tài khoản. Giữ từ 1 tuần đến 1 tháng để thành thói quen. Ba lỗi như 3 tảng đá trên đường. Quay lại. Hoặc vượt qua từng tảng 1. Bạn đang vướng lỗi nào? Theo dõi sốt trading để học giao dịch bên vững hơn.</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1:13</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7695191312605187348</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695389393443409173</t>
         </is>
       </c>
     </row>
@@ -2840,27 +2840,27 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Đầu tư và giao dịch khác nhau ở đâu? Đầu tư và giao dịch giống nhau ở...</t>
+          <t>Chứng khoán, tiền điện tử hay ngoại hối: chọn thị trường nào? So sánh...</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Đầu tư và giao dịch khác nhau ở đâu? Đầu tư và giao dịch giống nhau ở bản chất mua rẻ bán đắt, khác nhau ở thời gian giữ lệnh và tâm lý. Video giải thích ngắn gọn, dễ hiểu. #trading #fx #crypto</t>
+          <t>Chứng khoán, tiền điện tử hay ngoại hối: chọn thị trường nào? So sánh 3 thị trường theo 4 đặc điểm: pháp lý, thanh khoản, thời gian giao dịch, nền tảng. Nguồn: nội dung do tác giả cung cấp. #Shorts #trading #xuhuong #crypto #fx</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Đầu tư và giao dịch khác nhau ở đâu? Hầu hết mọi người đều hiểu sai, ở cả 3 thị trường, bản chất đều giống nhau, mua giá thấp, bán giá cao, chứng khoán, mua bán cổ phiếu, tức quyền sở hữu một phần công ty, tiền điện tử là Bitcoin và các đồng khác. Ngoại hối là Đô Là Mỹ, Yên Nhật khác nhau chính là thời gian giữ lệnh, giữ nhiều tháng, nhiều năm là đầu tư. Giữ theo food, giờ, ngay là giao dịch, đầu tư không tốn nhiều thời gian như giao dịch, nhưng vẫn mang lại nguồn thu nhập tốt, nhưng có người đầu tư mà nhìn giá cả ngày, lỗ thì mất ngủ. Đó là tâm lý giao dịch, ngược lại, có người giao dịch ít lệnh và đúng lúc vẫn có thời gian cho việc khác, che tên sản phẩm đi, chỉ còn nến và giá. Chọn thị trường theo đặc điểm, không phải vì biết nó trước, đầu tư hay giao dịch chỉ đa, kết quả nằm ở cách bạn dùng nó, theo dõi để học thêm nha.</t>
+          <t>Trứng khoán, tiền điện tử hay ngoại hối, chọn sai thị trường là mất tiền. Bối thị trường có đặc điểm riêng, hãy xét bốn thứ, pháp lý, thanh khoản, thời gian giao dịch và nền tảng. Pháp lý, trứng khoán được nhà nước bảo hộ chặt trẽ. Tiền điện tử và ngoại hối thì chưa được công nhận. Vì vậy, giữ số tiền lớn lâu dài thì trứng khoán an toàn hơn, đừng ném cả tài sản vào sản không tên tuổi. Thanh khoản, ngoại hối lớn nhất, rồi trứng khoán, rồi tiền điện tử. Nhưng trứng khoán Việt Nam thấp nhất nên chỉ hợp đầu tư dài hạn. Cổ phiếu và tiền điện tử dễ bị thao túng, biến động vài chục phần trăm. Cặp tiền lệch 1 phần trăm 1 ngày đã là nhiều. Thời gian, trứng khoán chỉ mở khoảng 4 tiếng 1 ngày, ngoại hối 24h, 5 ngày, tiền điện tử 24h, 7 ngày, nền tảng. Sanh ngoại hối giao dịch được tiền tệ, tiền điện tử, chỉ số và vàng. Nhưng đó là hợp đồng tranh lệch bạn không sở hữu tài sản. Tóm lại, trứng khoán hợp dài hạn, ngoại hối chỉ hợp ngắn hạn. Tiền điện tử hợp cả 2 nhưng rủi do cao, và dù chọn thị trường nào cũng phải chọn sản uy tín. Sanh kém thì ở đâu cũng dễ mất tiền, theo dõi để học cách bảo vệ và làm sinh lời đồng vốn của bạn mỗi ngày.</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>1:13</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694935798524742932</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7695191312605187348</t>
         </is>
       </c>
     </row>
@@ -2890,27 +2890,27 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>4 bước vào lệnh chuẩn: cấu trúc, khung lớn, vùng cản, tín hiệu yếu dầ...</t>
+          <t>Đầu tư và giao dịch khác nhau ở đâu? Đầu tư và giao dịch giống nhau ở...</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>4 bước vào lệnh chuẩn: cấu trúc, khung lớn, vùng cản, tín hiệu yếu dần Phương pháp vào lệnh gồm bốn bước kèm ví dụ ETHUSD khung M15. Nội dung do tác giả chia sẻ, không phải lời khuyên đầu tư.  #trading #fx #cypto</t>
+          <t>Đầu tư và giao dịch khác nhau ở đâu? Đầu tư và giao dịch giống nhau ở bản chất mua rẻ bán đắt, khác nhau ở thời gian giữ lệnh và tâm lý. Video giải thích ngắn gọn, dễ hiểu. #trading #fx #crypto</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Vào lệnh, đúng không phải đoán mò. Mà đi theo bốn bước. Bước 1, xác định cấu trúc trên khung đang giao dịch. Bước 2, tìm thêm yêu tố ủng hộ ở khung lớn hơn một bậc. Bước 3, chờ giá hồi về vùng cản quan trọng. Bước 4, chờ phê ngược lại yếu dần rồi mới vào lệnh. Ví dụ mua ATHSD 015, giá phá đỉnh 2 lần, đáy quan trọng vẫn được giữ. Chờ giá hồi về đỉnh cũ rồi mới mua, cắt lỗ dưới vùng đó. Lệnh lời gấp 3 rủi do, không xem thêm chỉ cần lớn hơn một bậc. 15 xem, 1, 1 xem, hư bốn, hư bốn xem khung ngày, cách này dùng được cho mọi thị trường. Khung lớn ủng hộ rõ, chỉ cần tín hiệu vừa phải ở khung nhỏ. Duyên đời mới chỉ là một chân của cái kiểu 3 chân. Theo rõi để xem 2 chân còn lại. Quán lý vốn và kỷ luật.</t>
+          <t>Đầu tư và giao dịch khác nhau ở đâu? Hầu hết mọi người đều hiểu sai, ở cả 3 thị trường, bản chất đều giống nhau, mua giá thấp, bán giá cao, chứng khoán, mua bán cổ phiếu, tức quyền sở hữu một phần công ty, tiền điện tử là Bitcoin và các đồng khác. Ngoại hối là Đô Là Mỹ, Yên Nhật khác nhau chính là thời gian giữ lệnh, giữ nhiều tháng, nhiều năm là đầu tư. Giữ theo food, giờ, ngay là giao dịch, đầu tư không tốn nhiều thời gian như giao dịch, nhưng vẫn mang lại nguồn thu nhập tốt, nhưng có người đầu tư mà nhìn giá cả ngày, lỗ thì mất ngủ. Đó là tâm lý giao dịch, ngược lại, có người giao dịch ít lệnh và đúng lúc vẫn có thời gian cho việc khác, che tên sản phẩm đi, chỉ còn nến và giá. Chọn thị trường theo đặc điểm, không phải vì biết nó trước, đầu tư hay giao dịch chỉ đa, kết quả nằm ở cách bạn dùng nó, theo dõi để học thêm nha.</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>51</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694847427051883796</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694935798524742932</t>
         </is>
       </c>
     </row>
@@ -2940,27 +2940,27 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Cách đọc cấu trúc thị trường: biết ngay phe mua hay phe bán thắng Các...</t>
+          <t>4 bước vào lệnh chuẩn: cấu trúc, khung lớn, vùng cản, tín hiệu yếu dầ...</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>Cách đọc cấu trúc thị trường: biết ngay phe mua hay phe bán thắng Cách đọc cấu trúc tăng, cấu trúc giảm và vùng đi ngang để biết nên mua, bán hay đứng ngoài. Nguồn: nội dung do tác giả cung cấp. #Shorts</t>
+          <t>4 bước vào lệnh chuẩn: cấu trúc, khung lớn, vùng cản, tín hiệu yếu dần Phương pháp vào lệnh gồm bốn bước kèm ví dụ ETHUSD khung M15. Nội dung do tác giả chia sẻ, không phải lời khuyên đầu tư.  #trading #fx #cypto</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Phần lớn người giao dịch thua lỗ chỉ vì một lý do. Không biết phê nào đang thắng, họ đổi phương pháp liên tục, vào lệnh theo cảm hứng và càng thua càng mất kiểm soát. Việc đầu tiên cần làm là biết lực mua hay lực bán đang chiếm ưu thế. Cấu chúc tăng là đáy sau cao hơn đáy trước. Đỉnh sau cao hơn đỉnh trước. Cấu chúc giảm thì ngược lại. Đỉnh thấp dần và đáy thấp dần. Hãy coi đó là một cuộc chiến. Mỗi đỉnh cũ là căn cứ của phê bán. Phê mua phá qua thì phê bán phải lùi. Một đáy chỉ quan trọng khi con sóng đi lên từ đáy đó phá qua đỉnh cũ. Phá qua, nghĩa là nến đóng cửa vượt qua. Râu nến quét rồi rút lại thì không tính. Giá nằm giữa đỉnh cao nhất và đáy quan trọng thì bị kẹp, thường đi ngang. Phá xuống đáy quan trọng cũng chưa phải xu hướng giảm. Chỉ khi giá hồi lên rồi phá tiếp đáy vừa tạo. xu hướng giảm mới được xác nhận. Cấu chúc tăng thì yêu tiên mua. Cấu chúc giảm thì yêu tiên bán. Còn rằng co thì đứng ngoài. Theo dõi để học thêm cách đọc thị trường.</t>
+          <t>Vào lệnh, đúng không phải đoán mò. Mà đi theo bốn bước. Bước 1, xác định cấu trúc trên khung đang giao dịch. Bước 2, tìm thêm yêu tố ủng hộ ở khung lớn hơn một bậc. Bước 3, chờ giá hồi về vùng cản quan trọng. Bước 4, chờ phê ngược lại yếu dần rồi mới vào lệnh. Ví dụ mua ATHSD 015, giá phá đỉnh 2 lần, đáy quan trọng vẫn được giữ. Chờ giá hồi về đỉnh cũ rồi mới mua, cắt lỗ dưới vùng đó. Lệnh lời gấp 3 rủi do, không xem thêm chỉ cần lớn hơn một bậc. 15 xem, 1, 1 xem, hư bốn, hư bốn xem khung ngày, cách này dùng được cho mọi thị trường. Khung lớn ủng hộ rõ, chỉ cần tín hiệu vừa phải ở khung nhỏ. Duyên đời mới chỉ là một chân của cái kiểu 3 chân. Theo rõi để xem 2 chân còn lại. Quán lý vốn và kỷ luật.</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694698536717356308</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694847427051883796</t>
         </is>
       </c>
     </row>
@@ -2990,27 +2990,27 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Học nhiều phương pháp vẫn mất tiền? Vì bạn chưa kiểm chứng Vì sao nhi...</t>
+          <t>Cách đọc cấu trúc thị trường: biết ngay phe mua hay phe bán thắng Các...</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Học nhiều phương pháp vẫn mất tiền? Vì bạn chưa kiểm chứng Vì sao nhiều người học phương pháp giao dịch vẫn thua lỗ, và cách kiểm chứng phương pháp bằng thống kê trước khi dùng tiền thật. #trading #crypto #btc #xuhuong</t>
+          <t>Cách đọc cấu trúc thị trường: biết ngay phe mua hay phe bán thắng Cách đọc cấu trúc tăng, cấu trúc giảm và vùng đi ngang để biết nên mua, bán hay đứng ngoài. Nguồn: nội dung do tác giả cung cấp. #Shorts</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Vì sao học nhiều phương pháp mà tài khoản vẫn cứ giảm, bạn tìm đủ loại phương pháp, cái nào nghe cũng hay như bí quyết, nhưng khi áp dụng thật, tài khoản cứ giảm dần vì có rất ít phương pháp thực sự đúng. Ngắn hạn, phương pháp nào cũng có lúc thắng lúc thua. Vào bừa cũng chỉ có 2 khả năng giá lên hoặc giá xuống. Vì vậy, hãy thống kê hàng trăm hàng nghìn lệnh. Nếu tỷ lệ thắng chỉ 50-50 thì chẳng khác gì may dùi. Hãy bỏ kiến thức chấp vá quay về biểu đồ giá. Mua giá thấp, bán giá cao hơn thì lời. Ngược lại thì lỗ, dù là chuyên gia hay người mới, lời hay lỗ cũng chỉ do giá. Hiểu cách giá di chuyển, bạn sẽ thấy quy luật, rút ra quý tắc, rồi kiểm trứng qua hàng trăm lệnh để biết tỷ lệ thắng và tỷ lệ lợi nhuận trên rủi do. Dùng tiền thật khi chưa kiểm trứng, giống như đi trong dừng mà không biết lối ra. Lộ trình đúng là tự nghiên cứu, thống kê kiểm trứng, rồi mới dùng tiền thật. Theo dõi kênh để học cách kiểm trứng phương pháp của riêng bạn.</t>
+          <t>Phần lớn người giao dịch thua lỗ chỉ vì một lý do. Không biết phê nào đang thắng, họ đổi phương pháp liên tục, vào lệnh theo cảm hứng và càng thua càng mất kiểm soát. Việc đầu tiên cần làm là biết lực mua hay lực bán đang chiếm ưu thế. Cấu chúc tăng là đáy sau cao hơn đáy trước. Đỉnh sau cao hơn đỉnh trước. Cấu chúc giảm thì ngược lại. Đỉnh thấp dần và đáy thấp dần. Hãy coi đó là một cuộc chiến. Mỗi đỉnh cũ là căn cứ của phê bán. Phê mua phá qua thì phê bán phải lùi. Một đáy chỉ quan trọng khi con sóng đi lên từ đáy đó phá qua đỉnh cũ. Phá qua, nghĩa là nến đóng cửa vượt qua. Râu nến quét rồi rút lại thì không tính. Giá nằm giữa đỉnh cao nhất và đáy quan trọng thì bị kẹp, thường đi ngang. Phá xuống đáy quan trọng cũng chưa phải xu hướng giảm. Chỉ khi giá hồi lên rồi phá tiếp đáy vừa tạo. xu hướng giảm mới được xác nhận. Cấu chúc tăng thì yêu tiên mua. Cấu chúc giảm thì yêu tiên bán. Còn rằng co thì đứng ngoài. Theo dõi để học thêm cách đọc thị trường.</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>59</t>
+          <t>58</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694588383363861781</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694698536717356308</t>
         </is>
       </c>
     </row>
@@ -3040,27 +3040,27 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Giá hồi cạn kiệt chưa? Cách chờ phe bán thất bại trước khi vào lệnh #...</t>
+          <t>Học nhiều phương pháp vẫn mất tiền? Vì bạn chưa kiểm chứng Vì sao nhi...</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Giá hồi cạn kiệt chưa? Cách chờ phe bán thất bại trước khi vào lệnh #Shorts Khi nào nhịp hồi trong xu hướng đã cạn kiệt để vào lệnh thuận xu hướng? Tóm tắt cách đọc lực mua bán bằng hành động giá: chờ phe bán thất bại 2–3 lần, có nến xác nhận rồi mới vào, đặt dừng lỗ dưới vùng cản và chốt lời ở vùng phe bán.</t>
+          <t>Học nhiều phương pháp vẫn mất tiền? Vì bạn chưa kiểm chứng Vì sao nhiều người học phương pháp giao dịch vẫn thua lỗ, và cách kiểm chứng phương pháp bằng thống kê trước khi dùng tiền thật. #trading #crypto #btc #xuhuong</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Giá vừa hồi về vùng cản bạn có nên mua ngay không? Câu trả lời thường là chưa. Giao dịch theo xu hướng nghĩa là, xu hướng tăng thì canh mua, xu hướng giảm thì canh bán. Nhưng không ai đuổi theo giá đã chạy xa vì càng đi xa, lực mua càng yếu dần. Bạn chỉ vào lệnh khi giá hồi và đồng thời phải hỏi. Nhịp hồi này đã cạn kiệt thật chưa? Hãy nhìn lực hay phè. Tại vùng cản phê mua, hối lượng mua lớn hơn bán nên giá bật lên. Nếu phê bán phá được vùng đó, nó thành vùng của phê bán. Và giá sẽ tiếp tục bị đẩy xuống. Dấu hiệu cạn kiệt là phê bán nhiều lần không phán nổi vùng giá. Hai đáy là lực bán giảm. Ba đáy kèm đến mua mạnh mới là cơ hội đẹp. Còn chưa có tín hiệu thì cứ đứng ngoài chờ. Đừng mua vội nếu điểm dừng lỗ quá xa hoặc điểm vào sát vùng cản của phê bán. Dừng lỗ dưới vùng cản phê mua, chốt lời ở vùng phê bán. Không có gì chắc chắn 100% thì bạn kiểm soát được là tỷ lệ thắng và tỷ lệ lợi nhuận trên rủi do. Kinh nhẫn trở phê, bán thất bại, theo dõi để học thêm cách độc lực mua bán và đừng vào lệnh khi nhịp hồi chưa cạn kiệt.</t>
+          <t>Vì sao học nhiều phương pháp mà tài khoản vẫn cứ giảm, bạn tìm đủ loại phương pháp, cái nào nghe cũng hay như bí quyết, nhưng khi áp dụng thật, tài khoản cứ giảm dần vì có rất ít phương pháp thực sự đúng. Ngắn hạn, phương pháp nào cũng có lúc thắng lúc thua. Vào bừa cũng chỉ có 2 khả năng giá lên hoặc giá xuống. Vì vậy, hãy thống kê hàng trăm hàng nghìn lệnh. Nếu tỷ lệ thắng chỉ 50-50 thì chẳng khác gì may dùi. Hãy bỏ kiến thức chấp vá quay về biểu đồ giá. Mua giá thấp, bán giá cao hơn thì lời. Ngược lại thì lỗ, dù là chuyên gia hay người mới, lời hay lỗ cũng chỉ do giá. Hiểu cách giá di chuyển, bạn sẽ thấy quy luật, rút ra quý tắc, rồi kiểm trứng qua hàng trăm lệnh để biết tỷ lệ thắng và tỷ lệ lợi nhuận trên rủi do. Dùng tiền thật khi chưa kiểm trứng, giống như đi trong dừng mà không biết lối ra. Lộ trình đúng là tự nghiên cứu, thống kê kiểm trứng, rồi mới dùng tiền thật. Theo dõi kênh để học cách kiểm trứng phương pháp của riêng bạn.</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1:03</t>
+          <t>59</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694492170773908757</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694588383363861781</t>
         </is>
       </c>
     </row>
@@ -3090,27 +3090,27 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Tìm vùng mua Bitcoin bằng cuộc chiến mua bán | Nến nhấn chìm + Fibona...</t>
+          <t>Giá hồi cạn kiệt chưa? Cách chờ phe bán thất bại trước khi vào lệnh #...</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Tìm vùng mua Bitcoin bằng cuộc chiến mua bán | Nến nhấn chìm + Fibonacci Cách đọc cuộc chiến phe mua - phe bán để tìm vùng mua Bitcoin, kết hợp nến nhấn chìm, Fibonacci và chia vốn nhiều giỏ.  #trading #crypto #btc</t>
+          <t>Giá hồi cạn kiệt chưa? Cách chờ phe bán thất bại trước khi vào lệnh #Shorts Khi nào nhịp hồi trong xu hướng đã cạn kiệt để vào lệnh thuận xu hướng? Tóm tắt cách đọc lực mua bán bằng hành động giá: chờ phe bán thất bại 2–3 lần, có nến xác nhận rồi mới vào, đặt dừng lỗ dưới vùng cản và chốt lời ở vùng phe bán.</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Bitcoin giảm sâu, nhưng có một vùng giá mà phê mua luôn lao vào. Bạn có biết nó nằm ở đâu không? Thì trường tiền điện tử chạy theo Bitcoin. Bitcoin chiếm phần lớn vốn hóa nên nó tăng thì cả thị trường tăng theo. Nguồn đọc giá, hãy nhìn cuộc chiến mua bán. Phê mua đẩy giá lên, rồi phê bán lại kéo giá xuống. Khi giá phá vùng cản của phê mua, phê bán chiếm yếu thế, hãy tìm vùng cản kế tiếp của phê mua nơi giá có thể bật lại. Phê bán thất bại nhiều lần, bóng đến dài kéo giá lên. Đây là dấu hiệu lực bán đang yếu dần, đừng vội vào lệnh. Hãy chờ tín hiệu rõ ràng, như cặp nên nhấn chìm tăng giá tại vùng cản mạnh. Vùng đó càng đáng tin khi chùng với mức Fibonacci của sống tăng trước đó. Các đồng lớn đều tạo tín hiệu tương tự. Sau khi đã giảm sâu từ 60 đến 70-3% mua ở vùng này, nếu giá giảm thêm thì bạn vẫn mua rẻ hơn người mua ở đỉnh. Giá quay lại đỉnh, bạn đã lại gấp đôi, đừng bỏ hết, vốn vào một giò. Chiếc vào nhiều đồng lớn, chỉ cần một đồng bay cao là đủ bù các đồng còn lại. Theo dõi để xem thêm phân tích mỗi ngày, đây không phải lời khuyên tài chính.</t>
+          <t>Giá vừa hồi về vùng cản bạn có nên mua ngay không? Câu trả lời thường là chưa. Giao dịch theo xu hướng nghĩa là, xu hướng tăng thì canh mua, xu hướng giảm thì canh bán. Nhưng không ai đuổi theo giá đã chạy xa vì càng đi xa, lực mua càng yếu dần. Bạn chỉ vào lệnh khi giá hồi và đồng thời phải hỏi. Nhịp hồi này đã cạn kiệt thật chưa? Hãy nhìn lực hay phè. Tại vùng cản phê mua, hối lượng mua lớn hơn bán nên giá bật lên. Nếu phê bán phá được vùng đó, nó thành vùng của phê bán. Và giá sẽ tiếp tục bị đẩy xuống. Dấu hiệu cạn kiệt là phê bán nhiều lần không phán nổi vùng giá. Hai đáy là lực bán giảm. Ba đáy kèm đến mua mạnh mới là cơ hội đẹp. Còn chưa có tín hiệu thì cứ đứng ngoài chờ. Đừng mua vội nếu điểm dừng lỗ quá xa hoặc điểm vào sát vùng cản của phê bán. Dừng lỗ dưới vùng cản phê mua, chốt lời ở vùng phê bán. Không có gì chắc chắn 100% thì bạn kiểm soát được là tỷ lệ thắng và tỷ lệ lợi nhuận trên rủi do. Kinh nhẫn trở phê, bán thất bại, theo dõi để học thêm cách độc lực mua bán và đừng vào lệnh khi nhịp hồi chưa cạn kiệt.</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1:05</t>
+          <t>1:03</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694281608039271701</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694492170773908757</t>
         </is>
       </c>
     </row>
@@ -3140,27 +3140,27 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Thị trường đi ngang: nhận biết &amp; tránh bị quét lệnh. #trading #fx #xu...</t>
+          <t>Tìm vùng mua Bitcoin bằng cuộc chiến mua bán | Nến nhấn chìm + Fibona...</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Thị trường đi ngang: nhận biết &amp; tránh bị quét lệnh. #trading #fx #xuhuong</t>
+          <t>Tìm vùng mua Bitcoin bằng cuộc chiến mua bán | Nến nhấn chìm + Fibonacci Cách đọc cuộc chiến phe mua - phe bán để tìm vùng mua Bitcoin, kết hợp nến nhấn chìm, Fibonacci và chia vốn nhiều giỏ.  #trading #crypto #btc</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>Lệnh của bạn hay bị quét. Thủ phạm chính là thị trường đi ngang. Thực tế không có lý thuyết nào xác định chính xác khi nào thị trường đi ngang. Nhưng có một cách dễ hiểu. Nhìn cuộc chiến giữa phê mua và phê bán. Phê mua phá đỉnh, phê bán phá đáy thì su hướng rõ ràng. Nhưng khi cả hai cùng thất bại, không ai chiêm yêu thế, thị trường bắt đầu đi ngang. Dấu hiệu nhận biết, ít nhất hai đỉnh và hai đáy ra cứ bật lại trong một hình chữ nhật. Thực tế, đỉnh đáy có thể lệch một chút. Giá phản ứng càng nhiều ở hai vùng cản thì vùng đi ngang cảng rõ. Chỉ khi một con sóng mạnh phá ra ngoài, một phê mới thật sự chiến thắng. Hãy chú ý biên độ. Nếu vùng đi ngang quá nhỏ so với sóng trước đó, su hướng cũ gần như không bị ảnh hưởng. Hãy nhìn khung thời gian lớn hơn. Đoạn trông như su hướng ở khung nhỏ có thể chỉ là một phần của vùng đi ngang ở khung H4 hay ngày. Ví dụ, giá hồi về vùng cản của phê bán, đỉnh thấp dần, rồi nến xanh phá vùng cản xác nhận lực bán đá cạn. Đó là điểm vào lệnh mua. Đặt cắt lỗ sau vùng cản, chốt lời ở các vùng cản kế tiếp và đừng chỉ chốt ở tỷ lệ một ăn một. Cần có lý do để kỳ vọng tỷ lệ cao hơn. Muốn xác xuất thắng cao. Hãy đứng ngoài khi thị trường đi ngang theo dõi để học thêm nhé!</t>
+          <t>Bitcoin giảm sâu, nhưng có một vùng giá mà phê mua luôn lao vào. Bạn có biết nó nằm ở đâu không? Thì trường tiền điện tử chạy theo Bitcoin. Bitcoin chiếm phần lớn vốn hóa nên nó tăng thì cả thị trường tăng theo. Nguồn đọc giá, hãy nhìn cuộc chiến mua bán. Phê mua đẩy giá lên, rồi phê bán lại kéo giá xuống. Khi giá phá vùng cản của phê mua, phê bán chiếm yếu thế, hãy tìm vùng cản kế tiếp của phê mua nơi giá có thể bật lại. Phê bán thất bại nhiều lần, bóng đến dài kéo giá lên. Đây là dấu hiệu lực bán đang yếu dần, đừng vội vào lệnh. Hãy chờ tín hiệu rõ ràng, như cặp nên nhấn chìm tăng giá tại vùng cản mạnh. Vùng đó càng đáng tin khi chùng với mức Fibonacci của sống tăng trước đó. Các đồng lớn đều tạo tín hiệu tương tự. Sau khi đã giảm sâu từ 60 đến 70-3% mua ở vùng này, nếu giá giảm thêm thì bạn vẫn mua rẻ hơn người mua ở đỉnh. Giá quay lại đỉnh, bạn đã lại gấp đôi, đừng bỏ hết, vốn vào một giò. Chiếc vào nhiều đồng lớn, chỉ cần một đồng bay cao là đủ bù các đồng còn lại. Theo dõi để xem thêm phân tích mỗi ngày, đây không phải lời khuyên tài chính.</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1:11</t>
+          <t>1:05</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694189318134369556</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694281608039271701</t>
         </is>
       </c>
     </row>
@@ -3190,27 +3190,27 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Lý thuyết Dow: vì sao vào lệnh theo sách vẫn thua? Lý thuyết Dow là n...</t>
+          <t>Thị trường đi ngang: nhận biết &amp; tránh bị quét lệnh. #trading #fx #xu...</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Lý thuyết Dow: vì sao vào lệnh theo sách vẫn thua? Lý thuyết Dow là nền móng của phân tích kỹ thuật, nhưng áp dụng quá cứng nhắc rất dễ thua. Video tóm tắt nhược điểm của định nghĩa xu hướng và cách hỏi "phe mua hay phe bán đang chiếm ưu thế" trước mỗi lệnh. #trading #fx #xuhuong</t>
+          <t>Thị trường đi ngang: nhận biết &amp; tránh bị quét lệnh. #trading #fx #xuhuong</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Học lý thuyết đào mà vào lệnh vẫn thua. Vấn đề nằm ở chỗ áp dụng quá cứng nhắc. Lý thuyết đào là nền móng của phân tích kỹ thuật. Nhưng chỉ thuộc định nghĩa thì chưa đủ để giao dịch. Theo sách, gia pha đáy quan trọng nghĩa là su hướng tăng đã đảo chiều thành giảm. Nhưng đáy nào mới là đáy quan trọng. Khung hết bốn và khung hết, một cho da hai đáy khác nhau. Nhiều khi bạn vội canh bán, giá lại chạm vùng cản của phê mua và bật tăng trở lại. Bởi phá đáy ở khung nhỏ chỉ cho thấy phê bán thắng một hiệp. Bức tranh lớn, phê mua vẫn mạnh hơn. Vậy hãy tự hỏi, lúc này phê mua hay phê bán đang chiếm yêu thế? Vẽ các vùng cản gần nhất của hai phê, rồi so sánh xóng giảm với xóng tăng trước đó. Phê mua còn mạnh thì canh mua ở vùng cản của phê mua đặt cắt lỗ bên dưới, chốt lời ở các vùng cản phía trên. Đừng áp dụng máy móc, theo dõi kênh để học cách vào lệnh theo su hướng hiệu quả.</t>
+          <t>Lệnh của bạn hay bị quét. Thủ phạm chính là thị trường đi ngang. Thực tế không có lý thuyết nào xác định chính xác khi nào thị trường đi ngang. Nhưng có một cách dễ hiểu. Nhìn cuộc chiến giữa phê mua và phê bán. Phê mua phá đỉnh, phê bán phá đáy thì su hướng rõ ràng. Nhưng khi cả hai cùng thất bại, không ai chiêm yêu thế, thị trường bắt đầu đi ngang. Dấu hiệu nhận biết, ít nhất hai đỉnh và hai đáy ra cứ bật lại trong một hình chữ nhật. Thực tế, đỉnh đáy có thể lệch một chút. Giá phản ứng càng nhiều ở hai vùng cản thì vùng đi ngang cảng rõ. Chỉ khi một con sóng mạnh phá ra ngoài, một phê mới thật sự chiến thắng. Hãy chú ý biên độ. Nếu vùng đi ngang quá nhỏ so với sóng trước đó, su hướng cũ gần như không bị ảnh hưởng. Hãy nhìn khung thời gian lớn hơn. Đoạn trông như su hướng ở khung nhỏ có thể chỉ là một phần của vùng đi ngang ở khung H4 hay ngày. Ví dụ, giá hồi về vùng cản của phê bán, đỉnh thấp dần, rồi nến xanh phá vùng cản xác nhận lực bán đá cạn. Đó là điểm vào lệnh mua. Đặt cắt lỗ sau vùng cản, chốt lời ở các vùng cản kế tiếp và đừng chỉ chốt ở tỷ lệ một ăn một. Cần có lý do để kỳ vọng tỷ lệ cao hơn. Muốn xác xuất thắng cao. Hãy đứng ngoài khi thị trường đi ngang theo dõi để học thêm nhé!</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>52</t>
+          <t>1:11</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7694116254126263573</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694189318134369556</t>
         </is>
       </c>
     </row>
@@ -3240,27 +3240,27 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Vai Đầu Vai: 3 dấu hiệu mô hình đẹp và 2 điểm vào lệnh #Shorts Cách c...</t>
+          <t>Lý thuyết Dow: vì sao vào lệnh theo sách vẫn thua? Lý thuyết Dow là n...</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Vai Đầu Vai: 3 dấu hiệu mô hình đẹp và 2 điểm vào lệnh #Shorts Cách chọn mô hình Vai Đầu Vai đẹp và hai điểm vào lệnh. Tóm ý từ video 'Phương Pháp Vào Lệnh Với Mô Hình VAI ĐẦU VAI Hoàn Hảo'</t>
+          <t>Lý thuyết Dow: vì sao vào lệnh theo sách vẫn thua? Lý thuyết Dow là nền móng của phân tích kỹ thuật, nhưng áp dụng quá cứng nhắc rất dễ thua. Video tóm tắt nhược điểm của định nghĩa xu hướng và cách hỏi "phe mua hay phe bán đang chiếm ưu thế" trước mỗi lệnh. #trading #fx #xuhuong</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Vài đầu vai nhìn đâu cũng thấy nhưng đa số vào lệnh sai ngay từ đầu. Vài đầu vai có 3 đỉnh, đỉnh giữa cao nhất, báo hiệu giá đảo chiều từ tăng sang giảm. Nhưng giá chỉ thật sự đảo chiều khi phá qua đường neckline, chưa phá thì phê bán chưa thắng. Dấu hiệu 1, các đỉnh trạm neckline phải nằm ngang nhau, không lệch quá nhiều. Dấu hiệu 2, vai phải càng gần neckline, phê bán càng yếu và điểm cắt lỗ càng gần. Dấu hiệu 3, mỗi bên có thể có nhiều vai, tranh chấp càng lâu thì cú phá càng đáng tin. Điểm vào thứ nhất, giá đóng cửa vượt neckline thì vào lệnh, cắt lỗ ở mức gần nhất. Điểm vào thứ 2, nếu nên phá quá dài, hãy chờ giá hồi về neckline dù mới vào, cẩn thận. Mô hình nhỏ nằm trong su hương lớn, ngược chiều rất dễ thất bại, hãy nhìn thêm vùng cản gần đó. Nếu giá chỉ chạy được 1 error thì bỏ qua, lưu lại 3 dấu hiệu này và theo dõi để học thêm. Nội dung chỉ mang tính giáo dục.</t>
+          <t>Học lý thuyết đào mà vào lệnh vẫn thua. Vấn đề nằm ở chỗ áp dụng quá cứng nhắc. Lý thuyết đào là nền móng của phân tích kỹ thuật. Nhưng chỉ thuộc định nghĩa thì chưa đủ để giao dịch. Theo sách, gia pha đáy quan trọng nghĩa là su hướng tăng đã đảo chiều thành giảm. Nhưng đáy nào mới là đáy quan trọng. Khung hết bốn và khung hết, một cho da hai đáy khác nhau. Nhiều khi bạn vội canh bán, giá lại chạm vùng cản của phê mua và bật tăng trở lại. Bởi phá đáy ở khung nhỏ chỉ cho thấy phê bán thắng một hiệp. Bức tranh lớn, phê mua vẫn mạnh hơn. Vậy hãy tự hỏi, lúc này phê mua hay phê bán đang chiếm yêu thế? Vẽ các vùng cản gần nhất của hai phê, rồi so sánh xóng giảm với xóng tăng trước đó. Phê mua còn mạnh thì canh mua ở vùng cản của phê mua đặt cắt lỗ bên dưới, chốt lời ở các vùng cản phía trên. Đừng áp dụng máy móc, theo dõi kênh để học cách vào lệnh theo su hướng hiệu quả.</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>52</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7693923604710378772</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7694116254126263573</t>
         </is>
       </c>
     </row>
@@ -3290,27 +3290,27 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>3 Bước Để Có Điểm Vào Lệnh Hoàn Hảo | Đọc Biểu Đồ Từ Khung Lớn Cách t...</t>
+          <t>Vai Đầu Vai: 3 dấu hiệu mô hình đẹp và 2 điểm vào lệnh #Shorts Cách c...</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>3 Bước Để Có Điểm Vào Lệnh Hoàn Hảo | Đọc Biểu Đồ Từ Khung Lớn Cách tìm điểm vào lệnh có nhiều yếu tố ủng hộ: từ khung ngày, H4 đến H1. Nội dung chỉ để học, không phải lời khuyên đầu tư. #trading #fx #crypto</t>
+          <t>Vai Đầu Vai: 3 dấu hiệu mô hình đẹp và 2 điểm vào lệnh #Shorts Cách chọn mô hình Vai Đầu Vai đẹp và hai điểm vào lệnh. Tóm ý từ video 'Phương Pháp Vào Lệnh Với Mô Hình VAI ĐẦU VAI Hoàn Hảo'</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Bạn vào lệnh đúng lúc mà vẫn thua. Vấn đề nằm ở chỗ này, điểm vào đẹp không đến từ một cây nén mà từ nhiều yếu tố cùng ủng hộ. Bước 1, nhìn khu ngài chỉ vẽ vùng cung cầu gần nhất. Một cây nén tăng quá mạnh thường không bền, đó là vùng bán tiềm năng. Bước 2, sang khung 4 giờ, chờ giá phá vùng cản bằng đến thân dài. Nên thân ngắn hay giúp chân thì cẩn thận rất dễ là phá giả. Bước 3, đừng đuổi giá, hãy chờ giá hồi về vùng rồi mới tìm tín hiệu. Mẫu nén đẹp chưa đủ, phải thấy bên kia lao vào rồi thất bại. Đừng dùng quá nhiều khung thời gian vì sẽ làm dối phân tích của bạn. Dừng lỗ đặt trên vùng cản, chốt lời mặc định khoảng 2 error. Đừng đặt chốt lời quá xa, chỉ cần thắng trên 50% là đã có lời. Lưu video lại và theo dõi để xem thêm cách đọc biểu đồ nhé.</t>
+          <t>Vài đầu vai nhìn đâu cũng thấy nhưng đa số vào lệnh sai ngay từ đầu. Vài đầu vai có 3 đỉnh, đỉnh giữa cao nhất, báo hiệu giá đảo chiều từ tăng sang giảm. Nhưng giá chỉ thật sự đảo chiều khi phá qua đường neckline, chưa phá thì phê bán chưa thắng. Dấu hiệu 1, các đỉnh trạm neckline phải nằm ngang nhau, không lệch quá nhiều. Dấu hiệu 2, vai phải càng gần neckline, phê bán càng yếu và điểm cắt lỗ càng gần. Dấu hiệu 3, mỗi bên có thể có nhiều vai, tranh chấp càng lâu thì cú phá càng đáng tin. Điểm vào thứ nhất, giá đóng cửa vượt neckline thì vào lệnh, cắt lỗ ở mức gần nhất. Điểm vào thứ 2, nếu nên phá quá dài, hãy chờ giá hồi về neckline dù mới vào, cẩn thận. Mô hình nhỏ nằm trong su hương lớn, ngược chiều rất dễ thất bại, hãy nhìn thêm vùng cản gần đó. Nếu giá chỉ chạy được 1 error thì bỏ qua, lưu lại 3 dấu hiệu này và theo dõi để học thêm. Nội dung chỉ mang tính giáo dục.</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>47</t>
+          <t>55</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7693801024087264533</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7693923604710378772</t>
         </is>
       </c>
     </row>
@@ -3340,27 +3340,27 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>3 bước tìm điểm vào lệnh đẹp trong trading Cách chọn điểm vào lệnh đơ...</t>
+          <t>3 Bước Để Có Điểm Vào Lệnh Hoàn Hảo | Đọc Biểu Đồ Từ Khung Lớn Cách t...</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>3 bước tìm điểm vào lệnh đẹp trong trading Cách chọn điểm vào lệnh đơn giản: nhìn cấu trúc thị trường, tìm vùng mua tiềm năng, chờ tín hiệu 3 giai đoạn. #trading #fx #crypto</t>
+          <t>3 Bước Để Có Điểm Vào Lệnh Hoàn Hảo | Đọc Biểu Đồ Từ Khung Lớn Cách tìm điểm vào lệnh có nhiều yếu tố ủng hộ: từ khung ngày, H4 đến H1. Nội dung chỉ để học, không phải lời khuyên đầu tư. #trading #fx #crypto</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Một điểm và lệnh đơn giản mà rất nhiều người bỏ qua. Bước 1, nhìn cấu chúc thị trường. Tăng, giảm, đi ngang có quy luật hoặc đi ngang không quy luật, đi ngang không quy luật thì đứng ngoài. Vì rất dễ bị quét lệnh. Bước 2, tìm vùng mua tiềm năng. Đó là đầu con sóng tăng và đỉnh cũ vừa bị phá. Nhưng nếu giá phá quá yếu hoặc phá xa rồi bị kéo về mạnh thì vùng đó không còn tốt. Khi Phi Bonacci không phải 5 hoặc không phải 6, 1, 8 trùng đỉnh cũ, đó là vùng đẹp. Bước 3, trở tín hiệu. Giá chạm vùng có thể đảo chiều, quét giả hoặc đi tiếp. Giai đoạn 1, lực bán yếu dần, nén giút chân, giai đoạn 2, tranh chấp, những cây, nén nhỏ, đi ngang. Giai đoạn 3, một nén tăng mạnh bứt phá, xác nhận xu hướng. Thếu một giai đoạn thì đứng ngoài, kiên nhẫn, quản lý vốn, kiểm tra lại nhiều lần. Ý hiệu ích thì nhấn thích và đăng ký nhé. Nội dung chỉ để học, không phải lời quên đầu tư.</t>
+          <t>Bạn vào lệnh đúng lúc mà vẫn thua. Vấn đề nằm ở chỗ này, điểm vào đẹp không đến từ một cây nén mà từ nhiều yếu tố cùng ủng hộ. Bước 1, nhìn khu ngài chỉ vẽ vùng cung cầu gần nhất. Một cây nén tăng quá mạnh thường không bền, đó là vùng bán tiềm năng. Bước 2, sang khung 4 giờ, chờ giá phá vùng cản bằng đến thân dài. Nên thân ngắn hay giúp chân thì cẩn thận rất dễ là phá giả. Bước 3, đừng đuổi giá, hãy chờ giá hồi về vùng rồi mới tìm tín hiệu. Mẫu nén đẹp chưa đủ, phải thấy bên kia lao vào rồi thất bại. Đừng dùng quá nhiều khung thời gian vì sẽ làm dối phân tích của bạn. Dừng lỗ đặt trên vùng cản, chốt lời mặc định khoảng 2 error. Đừng đặt chốt lời quá xa, chỉ cần thắng trên 50% là đã có lời. Lưu video lại và theo dõi để xem thêm cách đọc biểu đồ nhé.</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>47</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7693735707138854164</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7693801024087264533</t>
         </is>
       </c>
     </row>
@@ -3390,27 +3390,27 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Vùng cung cầu trong trading. #trading #fx #Shorts</t>
+          <t>3 bước tìm điểm vào lệnh đẹp trong trading Cách chọn điểm vào lệnh đơ...</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Vùng cung cầu trong trading. #trading #fx #Shorts</t>
+          <t>3 bước tìm điểm vào lệnh đẹp trong trading Cách chọn điểm vào lệnh đơn giản: nhìn cấu trúc thị trường, tìm vùng mua tiềm năng, chờ tín hiệu 3 giai đoạn. #trading #fx #crypto</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Bẽ vùng cầu càng nhiều đường, bạn càng thua nhiều hơn, vì sao vùng cầu là nơi phe mua thắng thế, còn vùng cung là nơi phe bán thắng thế. Psylum phổ biến là vẽ mọi đường ngang đi qua thật nhiều đỉnh và đáy. Cách này không có quy tắc, đường nào cũng đúng, nên bạn không thể giao dịch được. Cách đúng thứ nhất, chỉ vẽ những vùng gần giá hiện tại nhất. Thứ 2, vẽ từ điểm cao nhất hoặc thấp nhất của đỉnh và đáy. Thứ 3, giá rời vùng càng nhanh và mạnh, vùng đó càng mạnh, nhưng vùng mạnh cũng đừng vào bừa. Hay chờ tín hiệu nên rõ ràng rồi, mới vào lệnh. Ví dụ thực tế, khung lớn phá đỉnh đi lên, giá hồi về vùng cầu, rồi tạo tín hiệu mua, sau đó giá tăng mạnh và chạm mục tiêu chốt lời. Kênh nhẫn chờ tín hiệu giúp bạn tránh một lệnh thua, theo dõi để xem thêm cách đọc biểu đồ, nội dung chỉ để học hỏi, không phải lời khuyên đầu tư.</t>
+          <t>Một điểm và lệnh đơn giản mà rất nhiều người bỏ qua. Bước 1, nhìn cấu chúc thị trường. Tăng, giảm, đi ngang có quy luật hoặc đi ngang không quy luật, đi ngang không quy luật thì đứng ngoài. Vì rất dễ bị quét lệnh. Bước 2, tìm vùng mua tiềm năng. Đó là đầu con sóng tăng và đỉnh cũ vừa bị phá. Nhưng nếu giá phá quá yếu hoặc phá xa rồi bị kéo về mạnh thì vùng đó không còn tốt. Khi Phi Bonacci không phải 5 hoặc không phải 6, 1, 8 trùng đỉnh cũ, đó là vùng đẹp. Bước 3, trở tín hiệu. Giá chạm vùng có thể đảo chiều, quét giả hoặc đi tiếp. Giai đoạn 1, lực bán yếu dần, nén giút chân, giai đoạn 2, tranh chấp, những cây, nén nhỏ, đi ngang. Giai đoạn 3, một nén tăng mạnh bứt phá, xác nhận xu hướng. Thếu một giai đoạn thì đứng ngoài, kiên nhẫn, quản lý vốn, kiểm tra lại nhiều lần. Ý hiệu ích thì nhấn thích và đăng ký nhé. Nội dung chỉ để học, không phải lời quên đầu tư.</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>49</t>
+          <t>56</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7693564151402302740</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7693735707138854164</t>
         </is>
       </c>
     </row>
@@ -3440,27 +3440,27 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>2 mẫu nến đảo chiều đáng học: chòm râu &amp; nhấn chìm lần hai Đọc nến từ...</t>
+          <t>Vùng cung cầu trong trading. #trading #fx #Shorts</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>2 mẫu nến đảo chiều đáng học: chòm râu &amp; nhấn chìm lần hai Đọc nến từ bản chất mua – bán và 2 mẫu nến đảo chiều tại vùng cản. Nội dung chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #trading #fx</t>
+          <t>Vùng cung cầu trong trading. #trading #fx #Shorts</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Nên nhấn chìm xuất hiện là đảo chiều. Chưa chắc đâu, mỗi cây nén là một cuộc chiến giữa phê mua và phê bán. Nén có 5 yếu tố, giám mở, giá đóng, cao nhất, thấp nhất và thời gian. Sau một sóng tăng, nên nhấn chìm giảm chỉ là nhịp hồi. Lực mua vẫn còn bẫu thứ nhất. Nên chỏm râu, từ 3 cây có râu dài trở lên. Râu càng dài, thị trường càng từ chối giám mạnh tại vùng đó. Bẫu thứ 2, nên nhấn chìm mở đỉnh, hoặc đáy lần thứ 2, đừng vào ở lần chạm đầu, hãy đợi nến đóng cửa rồi mới hành động. Đặt cắt lỗ dưới râu nén hoặc dưới vùng cản để kiểm soát rủi do. Điểm vào tốt phải có quý tắc rõ ràng đến nơi chỉ việc kiểm tra. Hãy tự hỏi, phê nào đang mạnh hơn? Theo dõi để học thêm và nhớ đây chỉ là kiến thức giáo dục.</t>
+          <t>Bẽ vùng cầu càng nhiều đường, bạn càng thua nhiều hơn, vì sao vùng cầu là nơi phe mua thắng thế, còn vùng cung là nơi phe bán thắng thế. Psylum phổ biến là vẽ mọi đường ngang đi qua thật nhiều đỉnh và đáy. Cách này không có quy tắc, đường nào cũng đúng, nên bạn không thể giao dịch được. Cách đúng thứ nhất, chỉ vẽ những vùng gần giá hiện tại nhất. Thứ 2, vẽ từ điểm cao nhất hoặc thấp nhất của đỉnh và đáy. Thứ 3, giá rời vùng càng nhanh và mạnh, vùng đó càng mạnh, nhưng vùng mạnh cũng đừng vào bừa. Hay chờ tín hiệu nên rõ ràng rồi, mới vào lệnh. Ví dụ thực tế, khung lớn phá đỉnh đi lên, giá hồi về vùng cầu, rồi tạo tín hiệu mua, sau đó giá tăng mạnh và chạm mục tiêu chốt lời. Kênh nhẫn chờ tín hiệu giúp bạn tránh một lệnh thua, theo dõi để xem thêm cách đọc biểu đồ, nội dung chỉ để học hỏi, không phải lời khuyên đầu tư.</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>45</t>
+          <t>49</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7693471867973176596</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7693564151402302740</t>
         </is>
       </c>
     </row>
@@ -3490,27 +3490,27 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>#fx #crypto #trading #sotrading #fomc</t>
+          <t>2 mẫu nến đảo chiều đáng học: chòm râu &amp; nhấn chìm lần hai Đọc nến từ...</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>#fx #crypto #trading #sotrading #fomc</t>
+          <t>2 mẫu nến đảo chiều đáng học: chòm râu &amp; nhấn chìm lần hai Đọc nến từ bản chất mua – bán và 2 mẫu nến đảo chiều tại vùng cản. Nội dung chỉ mang tính giáo dục, không phải lời khuyên đầu tư. #Shorts #trading #fx</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Đã bao giờ bạn ngồi thẫn thờ trước màn hình lúc 3 giờ sáng, nhìn chân chân vào con số không tròn chính chưa? Ánh sáng đỏ từ nến sắp hắt lên khuôn mặt phở phạc, và hai bàn tay thì lạnh toát. Cảm giác đó, sự tuyệt vọng đến tột cùng. Bạn gục đầu xuống, tự tác vào mặt mình vì sự ngu ngốc. Tại sao không giết khoát cắt lỗ? Tại sao lại gun dày kéo dày? Tại sao lại mù quán ô lín bấu viếu vào một phép màu? Nhưng điều đâm nắt trái tim bạn không phải là những con số vô chi. Số tiền đó lẽ ra là tiền bìm sữa cho con. Bạn phải gượng cười, nuốt ngược cái hố sâu hấm vào dạ dày. Bạn thấy mình giống một kẻ lừa đảo thảm hại. Bạn gào thét đổ lỗi cho nhà cái quét râu. Nhưng sâu thằm, bạn biết rõ sự thật. Chẳng ai xan tìm bạn cả. Chính sự do dự bóp nghẹt stop loss đã tạo ra phịt tài khoản. Chính lòng tham của bạn đã tự tay châm ngòi nổ. Thị trường không có sự chắc ẩn. Lối thoát duy nhất là giết chết cảm xúc. Đánh như một cổ máy máu lạnh. Tự bóp chết cảm xúc. Hay để thị trường bóp chết bạn.</t>
+          <t>Nên nhấn chìm xuất hiện là đảo chiều. Chưa chắc đâu, mỗi cây nén là một cuộc chiến giữa phê mua và phê bán. Nén có 5 yếu tố, giám mở, giá đóng, cao nhất, thấp nhất và thời gian. Sau một sóng tăng, nên nhấn chìm giảm chỉ là nhịp hồi. Lực mua vẫn còn bẫu thứ nhất. Nên chỏm râu, từ 3 cây có râu dài trở lên. Râu càng dài, thị trường càng từ chối giám mạnh tại vùng đó. Bẫu thứ 2, nên nhấn chìm mở đỉnh, hoặc đáy lần thứ 2, đừng vào ở lần chạm đầu, hãy đợi nến đóng cửa rồi mới hành động. Đặt cắt lỗ dưới râu nén hoặc dưới vùng cản để kiểm soát rủi do. Điểm vào tốt phải có quý tắc rõ ràng đến nơi chỉ việc kiểm tra. Hãy tự hỏi, phê nào đang mạnh hơn? Theo dõi để học thêm và nhớ đây chỉ là kiến thức giáo dục.</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>45</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7687234989431278868</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7693471867973176596</t>
         </is>
       </c>
     </row>
@@ -3540,27 +3540,27 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>#trading #cpi #sotrading #crypto #fx</t>
+          <t>#fx #crypto #trading #sotrading #fomc</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>#trading #cpi #sotrading #crypto #fx</t>
+          <t>#fx #crypto #trading #sotrading #fomc</t>
         </is>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn</t>
+          <t>Đã bao giờ bạn ngồi thẫn thờ trước màn hình lúc 3 giờ sáng, nhìn chân chân vào con số không tròn chính chưa? Ánh sáng đỏ từ nến sắp hắt lên khuôn mặt phở phạc, và hai bàn tay thì lạnh toát. Cảm giác đó, sự tuyệt vọng đến tột cùng. Bạn gục đầu xuống, tự tác vào mặt mình vì sự ngu ngốc. Tại sao không giết khoát cắt lỗ? Tại sao lại gun dày kéo dày? Tại sao lại mù quán ô lín bấu viếu vào một phép màu? Nhưng điều đâm nắt trái tim bạn không phải là những con số vô chi. Số tiền đó lẽ ra là tiền bìm sữa cho con. Bạn phải gượng cười, nuốt ngược cái hố sâu hấm vào dạ dày. Bạn thấy mình giống một kẻ lừa đảo thảm hại. Bạn gào thét đổ lỗi cho nhà cái quét râu. Nhưng sâu thằm, bạn biết rõ sự thật. Chẳng ai xan tìm bạn cả. Chính sự do dự bóp nghẹt stop loss đã tạo ra phịt tài khoản. Chính lòng tham của bạn đã tự tay châm ngòi nổ. Thị trường không có sự chắc ẩn. Lối thoát duy nhất là giết chết cảm xúc. Đánh như một cổ máy máu lạnh. Tự bóp chết cảm xúc. Hay để thị trường bóp chết bạn.</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1:10</t>
+          <t>50</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7686468492828331285</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7687234989431278868</t>
         </is>
       </c>
     </row>
@@ -3590,17 +3590,17 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>#trading #cpi #fx #sotrading #crypto</t>
+          <t>#trading #cpi #sotrading #crypto #fx</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>#trading #cpi #fx #sotrading #crypto</t>
+          <t>#trading #cpi #sotrading #crypto #fx</t>
         </is>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Cùng nhận một tín hiệu. Tại sao mỗi người lại có một kết quả khác nhau? Ba người cùng nhận được một tín hiệu với đầy đủ điểm vào, điểm dừng và mục tiêu. Người đầu tiên thực hiện đúng vùng giá, chọn khối lượng phù hợp và chỉ chấp nhận mức dùi do đã tính trước. Người thứ 2 xem tín hiệu muộn. Giá đã chạy khỏi vùng vào nhưng vì sợ bỏ lỡ nên vẫn quyết định tham gia. Người thứ 3 thấy cơ hội hấp dẫn nên tự ý tăng khối lượng lên nhiều lần. Khi thị trường biến động ngược hướng, người đầu chịu đúng dùi do trong kế hoạch, người thứ 2 tổn thất lớn, còn người thứ 3 chạm giấy hạn, thổi bay tài khoản. Như vậy, vấn đề không chỉ nằm ở tín hiệu. Cùng một tín hiệu, nhưng điểm vào, khối lượng và cách kiểm soát dùi do khác nhau sẽ tạo ra kết quả hoàn toàn khác nhau. Đó là lý do mình phát triển hệ thống tiếp nhận và thực thi tín hiệu tự động. Hệ thống hỗ trợ thiết lập điểm vào, điểm dừng, mục tiêu và khối lượng chuẩn sát dựa trên mức dùi do bạn đã cài. Hệ thống không hứa hẹn mọi lệnh đều thắng. Mục tiêu là hạn chế sai sót và ép bạn tuân thủ, tín hiệu, tín hiệu tạo cơ hội, nhưng thực hiện quyết định kết quả, bạn hay gặp vấn đề điểm vào, khối lượng hay cảm xúc, bình luận để xem hệ thống hoạt động nhá.</t>
+          <t>Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn Hãy subscribe cho kênh Ghiền Mì Gõ Để không bỏ lỡ những video hấp dẫn</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -3610,7 +3610,7 @@
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7686097369682922772</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7686468492828331285</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3650,7 @@
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Nếu tay bạn dùn lên và nhịp tim đập thỉnh thịch mỗi khi bấm lệnh, thì hãy rút sạch tiền và xóa áp đi. Bạn không phải là một trader, bạn đang tự nguyện bước vào lò mổ. Mạng xã hội đã lừa rối bạn, những video khoe siêu xe, những cú chốt lời xanh mướt x5 x10 tài khoản chỉ sau một đêm. Đó chỉ là mồi nhử và sự tham laam của bạn, chính là chiếc lưỡi câu. Họ làm bạn nghiện cái cảm giác nghẹt thờ, Nghiện lượng hốc môn kích thích bơm thẳng lên áo mỗi khi nến rật lên rật xuống, mắt bạn rán chặt vào màn hình trường đường quest stop lot. Bạn tưởng mình đang phân bằng chính những đồng áo máu của gia đình mình. Và đây là sự thật tàn nhẫn nhất mà đám thầy bà ngoài kia không bao giờ dám nói cho bạn biết. Một hệ thống giao dịch thực sự kiếm được tiền nó tẻ nhạt đến mức đáng sợ. Đúng vậy, chán ngắt. Trong khi bạn đang gào thét, đập bàn đập ghế vì một lệnh lỗ, thì những kẻ đang âm thầm lấy tiền của bạn ngoài kia. Họ vô cảm. Họ coi tiền trên màn hình chỉ là con số, đó là trò chơi của sắc xuất. Kỳ luật không phải gồng mình chịu đựng, nó là cố máy máu lạnh, không hy vọng, cũng không có sợ hãi, nhạt nhéo như việc bạn đánh dăng. Đã đến lúc bạn phải lựa chọn, hoặc là tự tay bóp chết cảm xúc và ảo tưởng của mình. Hoặc là để thị trường nhai nát tài khoản của bạn và nhổ ra không thương tiếc.</t>
+          <t>Cùng nhận một tín hiệu. Tại sao mỗi người lại có một kết quả khác nhau? Ba người cùng nhận được một tín hiệu với đầy đủ điểm vào, điểm dừng và mục tiêu. Người đầu tiên thực hiện đúng vùng giá, chọn khối lượng phù hợp và chỉ chấp nhận mức dùi do đã tính trước. Người thứ 2 xem tín hiệu muộn. Giá đã chạy khỏi vùng vào nhưng vì sợ bỏ lỡ nên vẫn quyết định tham gia. Người thứ 3 thấy cơ hội hấp dẫn nên tự ý tăng khối lượng lên nhiều lần. Khi thị trường biến động ngược hướng, người đầu chịu đúng dùi do trong kế hoạch, người thứ 2 tổn thất lớn, còn người thứ 3 chạm giấy hạn, thổi bay tài khoản. Như vậy, vấn đề không chỉ nằm ở tín hiệu. Cùng một tín hiệu, nhưng điểm vào, khối lượng và cách kiểm soát dùi do khác nhau sẽ tạo ra kết quả hoàn toàn khác nhau. Đó là lý do mình phát triển hệ thống tiếp nhận và thực thi tín hiệu tự động. Hệ thống hỗ trợ thiết lập điểm vào, điểm dừng, mục tiêu và khối lượng chuẩn sát dựa trên mức dùi do bạn đã cài. Hệ thống không hứa hẹn mọi lệnh đều thắng. Mục tiêu là hạn chế sai sót và ép bạn tuân thủ, tín hiệu, tín hiệu tạo cơ hội, nhưng thực hiện quyết định kết quả, bạn hay gặp vấn đề điểm vào, khối lượng hay cảm xúc, bình luận để xem hệ thống hoạt động nhá.</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -3660,7 +3660,7 @@
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7685719795400051989</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7686097369682922772</t>
         </is>
       </c>
     </row>
@@ -3690,17 +3690,17 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>#trading #cpi #trading #fx #sotrading</t>
+          <t>#trading #cpi #fx #sotrading #crypto</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>#trading #cpi #trading #fx #sotrading</t>
+          <t>#trading #cpi #fx #sotrading #crypto</t>
         </is>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>99% trầy trái tài khoản không phải vì rốt kỹ thuật, cũng chẳng phải vì thị trường cố tình đi ngược lại họ. Lý do thực sự là vì tất cả chúng ta đều từng mắc kẹt trong một áo tưởng điên cuồng, đi tìm một chén thánh giao dịch. Kịch bản này quen không? Nạp tiền, ăn vài lệnh đầu, bạn tự tin tháo stoplots vì cay cũ, để rồi tài khoản trái khét, sáng ra với đầu chống rỗng, vòng xoay đó cứ lập lại. Tại sao? Vì tư duy của bạn chưa thay đổi, bạn không chấp nhận mình có thể sai, bạn ảo tưởng nhồi nhét thêm vài chỉ báo là kiểm soát được thị trường, tỉnh lại đi, bạn sẽ bị nó nghiền nát. Nhiều người cậy mình có kỹ năng, họ stoplots lại thật hẹp, phí giao dịch sẽ ăn món hết, khoản phí này mới là lưỡi giao, nó lặng lặng gióc thịt tài khoản, chứ không phải do nhà cái. Ở thị trường này, sự thật mất lòng nhất là không có gì là tuyệt đối, và cũng chẳng có chén thánh nào cứu được bạn, lối thoát duy nhất để tồn tại và bất phá chỉ gói gọn trong hai chữ, từ duy và kỷ luật. Hãy học cách chấp nhận dùi do, trở thành người quản trị vốn tàn nhẫn, giao dịch là bài toán sắc xuất, kiểm soát nghiêm ngặt số tiền sẽ mất, để không bị đá vang khỏi cuộc chơi. Đừng để thị trường biến bạn thành một con bạc khát nước và tước đi sự tự tôn cuối cùng của mình. Khi sự hương phấn tột độ, hay nỗi sợ hãi tột cùng ập đến, thì kỷ luật chính là chiếc mỏ neo duy nhất giữ bạn lại với cuộc chơi.</t>
+          <t>Nếu tay bạn dùn lên và nhịp tim đập thỉnh thịch mỗi khi bấm lệnh, thì hãy rút sạch tiền và xóa áp đi. Bạn không phải là một trader, bạn đang tự nguyện bước vào lò mổ. Mạng xã hội đã lừa rối bạn, những video khoe siêu xe, những cú chốt lời xanh mướt x5 x10 tài khoản chỉ sau một đêm. Đó chỉ là mồi nhử và sự tham laam của bạn, chính là chiếc lưỡi câu. Họ làm bạn nghiện cái cảm giác nghẹt thờ, Nghiện lượng hốc môn kích thích bơm thẳng lên áo mỗi khi nến rật lên rật xuống, mắt bạn rán chặt vào màn hình trường đường quest stop lot. Bạn tưởng mình đang phân bằng chính những đồng áo máu của gia đình mình. Và đây là sự thật tàn nhẫn nhất mà đám thầy bà ngoài kia không bao giờ dám nói cho bạn biết. Một hệ thống giao dịch thực sự kiếm được tiền nó tẻ nhạt đến mức đáng sợ. Đúng vậy, chán ngắt. Trong khi bạn đang gào thét, đập bàn đập ghế vì một lệnh lỗ, thì những kẻ đang âm thầm lấy tiền của bạn ngoài kia. Họ vô cảm. Họ coi tiền trên màn hình chỉ là con số, đó là trò chơi của sắc xuất. Kỳ luật không phải gồng mình chịu đựng, nó là cố máy máu lạnh, không hy vọng, cũng không có sợ hãi, nhạt nhéo như việc bạn đánh dăng. Đã đến lúc bạn phải lựa chọn, hoặc là tự tay bóp chết cảm xúc và ảo tưởng của mình. Hoặc là để thị trường nhai nát tài khoản của bạn và nhổ ra không thương tiếc.</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7685348661768899860</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7685719795400051989</t>
         </is>
       </c>
     </row>
@@ -3740,27 +3740,27 @@
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>#trading #crypto #fx #cpi #sotrading</t>
+          <t>#trading #cpi #trading #fx #sotrading</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>#trading #crypto #fx #cpi #sotrading</t>
+          <t>#trading #cpi #trading #fx #sotrading</t>
         </is>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Sang tuần thứ 4, sự bế tắc đã biến A từ một người phân tích cẩn trọng thành một con bạc khát nước. Cậu không còn nhìn biểu đồ để tìm dòng tiền nữa. Cậu nhìn nó bằng ánh mắt của kẻ muốn trả thù. 10 giờ tối, một cây nến xanh bất phá, chỉ một lệnh all in này thôi. Gỡ lại 10.000 đô rồi mình sẽ đánh kỷ luật. A kéo tối đa đòn 7, nhắm mắt bấm bay và giết khoát tháo luôn stop loss. 5 phút đầu, tài khoản xanh mướt. Nhưng rồi giá khượng lại, đến giút chân đỏ quạch đâm xuống, phá vỡ mọi hỗ trợ. A chết lặng, mùa hôi lạnh túa ra, cậu cầu nguyện, cậu rán mắt vào những con số âm. Âm 1 ngàn dưới, âm 3 ngàn, âm 5 ngàn dưới, thanh lý hiện lên lạnh léo. Căn phòng rơi vào tính lặng. Không có tiếng gạo thét, chỉ có sự chống rõm tột cùng. Tại sao không cắt lỗ lúc nãy? Đêm đó, A mất ngủ, tự thể độc sẽ không bao giờ lặp lại. Nhưng bị kịch lớn nhất không phải là mất 10.000 đô. Vì gốc dễ tư duy chưa hề đập đi xay lại, bàn tay A lại tiếp tục bóp ngắn xóa điện ngục lại bắt đầu quay. Cuốn đi tất cả trong thị trường này, danh giới giữa một trader và một con bạc mỏng manh đến đáng sợ. Có thể bạn đang cười A, nhưng đã bao giờ bạn thấy bóng dáng mình trong đó. Còn anh em, anh em nhìn nhận thế nào về nhân vật A, hãy để lại ý kiến xuống phật bình luận nhé.</t>
+          <t>99% trầy trái tài khoản không phải vì rốt kỹ thuật, cũng chẳng phải vì thị trường cố tình đi ngược lại họ. Lý do thực sự là vì tất cả chúng ta đều từng mắc kẹt trong một áo tưởng điên cuồng, đi tìm một chén thánh giao dịch. Kịch bản này quen không? Nạp tiền, ăn vài lệnh đầu, bạn tự tin tháo stoplots vì cay cũ, để rồi tài khoản trái khét, sáng ra với đầu chống rỗng, vòng xoay đó cứ lập lại. Tại sao? Vì tư duy của bạn chưa thay đổi, bạn không chấp nhận mình có thể sai, bạn ảo tưởng nhồi nhét thêm vài chỉ báo là kiểm soát được thị trường, tỉnh lại đi, bạn sẽ bị nó nghiền nát. Nhiều người cậy mình có kỹ năng, họ stoplots lại thật hẹp, phí giao dịch sẽ ăn món hết, khoản phí này mới là lưỡi giao, nó lặng lặng gióc thịt tài khoản, chứ không phải do nhà cái. Ở thị trường này, sự thật mất lòng nhất là không có gì là tuyệt đối, và cũng chẳng có chén thánh nào cứu được bạn, lối thoát duy nhất để tồn tại và bất phá chỉ gói gọn trong hai chữ, từ duy và kỷ luật. Hãy học cách chấp nhận dùi do, trở thành người quản trị vốn tàn nhẫn, giao dịch là bài toán sắc xuất, kiểm soát nghiêm ngặt số tiền sẽ mất, để không bị đá vang khỏi cuộc chơi. Đừng để thị trường biến bạn thành một con bạc khát nước và tước đi sự tự tôn cuối cùng của mình. Khi sự hương phấn tột độ, hay nỗi sợ hãi tột cùng ập đến, thì kỷ luật chính là chiếc mỏ neo duy nhất giữ bạn lại với cuộc chơi.</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>1:11</t>
+          <t>1:10</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>https://www.tiktok.com/@sotrading01/video/7684604753577495829</t>
+          <t>https://www.tiktok.com/@sotrading01/video/7685348661768899860</t>
         </is>
       </c>
     </row>
@@ -3790,25 +3790,75 @@
       </c>
       <c r="F45" t="inlineStr">
         <is>
+          <t>#trading #crypto #fx #cpi #sotrading</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>#trading #crypto #fx #cpi #sotrading</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Sang tuần thứ 4, sự bế tắc đã biến A từ một người phân tích cẩn trọng thành một con bạc khát nước. Cậu không còn nhìn biểu đồ để tìm dòng tiền nữa. Cậu nhìn nó bằng ánh mắt của kẻ muốn trả thù. 10 giờ tối, một cây nến xanh bất phá, chỉ một lệnh all in này thôi. Gỡ lại 10.000 đô rồi mình sẽ đánh kỷ luật. A kéo tối đa đòn 7, nhắm mắt bấm bay và giết khoát tháo luôn stop loss. 5 phút đầu, tài khoản xanh mướt. Nhưng rồi giá khượng lại, đến giút chân đỏ quạch đâm xuống, phá vỡ mọi hỗ trợ. A chết lặng, mùa hôi lạnh túa ra, cậu cầu nguyện, cậu rán mắt vào những con số âm. Âm 1 ngàn dưới, âm 3 ngàn, âm 5 ngàn dưới, thanh lý hiện lên lạnh léo. Căn phòng rơi vào tính lặng. Không có tiếng gạo thét, chỉ có sự chống rõm tột cùng. Tại sao không cắt lỗ lúc nãy? Đêm đó, A mất ngủ, tự thể độc sẽ không bao giờ lặp lại. Nhưng bị kịch lớn nhất không phải là mất 10.000 đô. Vì gốc dễ tư duy chưa hề đập đi xay lại, bàn tay A lại tiếp tục bóp ngắn xóa điện ngục lại bắt đầu quay. Cuốn đi tất cả trong thị trường này, danh giới giữa một trader và một con bạc mỏng manh đến đáng sợ. Có thể bạn đang cười A, nhưng đã bao giờ bạn thấy bóng dáng mình trong đó. Còn anh em, anh em nhìn nhận thế nào về nhân vật A, hãy để lại ý kiến xuống phật bình luận nhé.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>1:11</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>https://www.tiktok.com/@sotrading01/video/7684604753577495829</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>🟢 Ưu tiên 3 (Thực chiến Price Action)</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>SO Trading</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>#cpi #sotrading #trading #fx #crypto</t>
         </is>
       </c>
-      <c r="G45" t="inlineStr">
+      <c r="G46" t="inlineStr">
         <is>
           <t>#cpi #sotrading #trading #fx #crypto</t>
         </is>
       </c>
-      <c r="H45" t="inlineStr">
+      <c r="H46" t="inlineStr">
         <is>
           <t>không phải là một kẻ ngốc. Trước khi nạp 10.000 đô đầu tiên, cậu đã dành hàng tháng trời cày nát các mô hình price action. Bước vào thị trường với một sự tự tin đầy tính toán. Những tuần đầu tiên, tiền nổ liên hồi. Cảm giác hoác môn hương phấn tiết ra tột độ khiến A bắt đầu tin rằng, mình sinh ra là để làm trader. Để tối đa hóa tỷ lệ lợi nhuận rùi do, ABOV STOP LOST lại thật hẹp. Cậu tự hào khoe những lệnh bắt đỉnh đáy như một phù thủy tài chính. Nhưng tuần trang mật kết thúc nhanh chóng. Giá vừa liếm S lờ thì ngay lập tức quay đầu bay đúng hướng. A, cây cú đập bàn, lũ nhà cái lại cố tình quét dâu mình. Cậu không hề nhận ra sự thật tàn nhẫn khoảng cách entry và S lờ quá ngắn khiến tỷ lệ phí giao dịch phình to khổng lồ vào cậu. Chính lưỡi giao vô hình của phí ẩn đang lặng lặng giọc thịt tài khoản. Tài khoản rơi từ 10.000 xuống 7.000 đô. Sự tự tin biến mất, nỗi sợ lên ngôi. Thay vì giữ kỷ luật 1% gốc, A run tay hạ cửa chỉ dám đánh 70 đô cho lệnh tiếp theo. Cái bẫy chính thức sập xuống, sai thì mất liên tục, mà đúng thì 140 đô thu về chỉ như cho đùa trước hố sâu 3.000 đô đang vẫn gì máu. Liệu A có kịp nhận ra nút thắt trước khi tài khoản vệch.</t>
         </is>
       </c>
-      <c r="I45" t="inlineStr">
+      <c r="I46" t="inlineStr">
         <is>
           <t>1:09</t>
         </is>
       </c>
-      <c r="J45" t="inlineStr">
+      <c r="J46" t="inlineStr">
         <is>
           <t>https://www.tiktok.com/@sotrading01/video/7684276294971854101</t>
         </is>

</xml_diff>